<commit_message>
Ses sistemi (SS1) kablosu 10 mm² olarak sabitlendi; ΔU aşımı uyarı ve bilinen sapma olarak raporlandı
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NjS5sn9fPFLq7X5eqGJ5mC
</commit_message>
<xml_diff>
--- a/cikti/04_hesap_tablolari.xlsx
+++ b/cikti/04_hesap_tablolari.xlsx
@@ -538,7 +538,7 @@
     <t xml:space="preserve">W18</t>
   </si>
   <si>
-    <t xml:space="preserve">NYY 3x25 mm² Cu</t>
+    <t xml:space="preserve">NYY 3x10 mm² Cu</t>
   </si>
   <si>
     <t xml:space="preserve">W19</t>
@@ -1195,7 +1195,7 @@
     <t xml:space="preserve">NYY 3x2,5 mm² Cu, L=28,0 m</t>
   </si>
   <si>
-    <t xml:space="preserve">NYY 3x25 mm² Cu, L=300,0 m</t>
+    <t xml:space="preserve">NYY 3x10 mm² Cu, L=300,0 m</t>
   </si>
   <si>
     <t xml:space="preserve">W19, W20</t>
@@ -5297,7 +5297,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
         <v>154</v>
       </c>
@@ -6127,7 +6127,7 @@
         <v>167</v>
       </c>
       <c r="J33" s="27" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="K33" s="27" t="n">
         <v>300</v>
@@ -6143,19 +6143,19 @@
       </c>
       <c r="O33" s="8" t="n">
         <f aca="false">INDEX($X$4:$Z$14,MATCH(J33,$W$4:$W$14,0),MATCH(L33,$X$3:$Z$3,0))</f>
-        <v>101</v>
+        <v>57</v>
       </c>
       <c r="P33" s="12" t="n">
         <f aca="false">O33*IF(L33="D2-3",$D$8,$D$7)</f>
-        <v>80.8</v>
+        <v>45.6</v>
       </c>
       <c r="Q33" s="11" t="n">
         <f aca="false">IF(F33="3F",SQRT(3),2)*H33*K33*AA33*(G33/($D$3*J33)+($D$4/1000)*SQRT(1-G33^2))</f>
-        <v>4.45071135511379</v>
+        <v>10.8538734104498</v>
       </c>
       <c r="R33" s="11" t="n">
         <f aca="false">Q33/IF(F33="3F",$D$5,$D$6)*100</f>
-        <v>1.93509189352774</v>
+        <v>4.71907539584772</v>
       </c>
       <c r="S33" s="11" t="n">
         <f aca="false">$R$15</f>
@@ -6163,7 +6163,7 @@
       </c>
       <c r="T33" s="11" t="n">
         <f aca="false">R33+S33</f>
-        <v>2.2073106917826</v>
+        <v>4.99129419410259</v>
       </c>
       <c r="U33" s="11" t="n">
         <f aca="false">IF(D33="aydınlatma",$D$10,$D$9)</f>
@@ -6171,7 +6171,7 @@
       </c>
       <c r="V33" s="24" t="str">
         <f aca="false">IF(AND(H33&lt;=N33,N33&lt;=P33,T33&lt;=U33),"UYGUN","UYGUN DEĞİL")</f>
-        <v>UYGUN</v>
+        <v>UYGUN DEĞİL</v>
       </c>
       <c r="AA33" s="9" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Çizim 6: ses kolları (SS1-SS3) güzergâhı, hoparlör uçları ve tablo satırları eklendi
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NjS5sn9fPFLq7X5eqGJ5mC
</commit_message>
<xml_diff>
--- a/cikti/04_hesap_tablolari.xlsx
+++ b/cikti/04_hesap_tablolari.xlsx
@@ -3181,7 +3181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
         <v>45</v>
       </c>
@@ -3229,7 +3229,7 @@
         <v>1.15942028985507</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
         <v>47</v>
       </c>
@@ -5647,7 +5647,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
         <v>162</v>
       </c>
@@ -5727,7 +5727,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
         <v>163</v>
       </c>
@@ -7532,7 +7532,7 @@
         <v>191</v>
       </c>
       <c r="F43" s="22" t="s">
-        <v>195</v>
+        <v>287</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7552,7 +7552,7 @@
         <v>191</v>
       </c>
       <c r="F44" s="22" t="s">
-        <v>195</v>
+        <v>287</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8302,7 +8302,7 @@
         <v>335</v>
       </c>
       <c r="F82" s="22" t="s">
-        <v>346</v>
+        <v>356</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Ses kollarına kol başına 4 hoparlör (HP1-HP12): poz kaydı, Çizim 1/6, Excel envanteri ve rapor güncellendi
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NjS5sn9fPFLq7X5eqGJ5mC
</commit_message>
<xml_diff>
--- a/cikti/04_hesap_tablolari.xlsx
+++ b/cikti/04_hesap_tablolari.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1194" uniqueCount="639">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1227" uniqueCount="651">
   <si>
     <t xml:space="preserve">YÜK DENGESİ VE FAZ DENGESİZLİĞİ</t>
   </si>
@@ -1171,6 +1171,27 @@
     <t xml:space="preserve">100 W, hat PJ3</t>
   </si>
   <si>
+    <t xml:space="preserve">HP1–HP4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hoparlör (ses kolu, hat gerilimli/doğrudan)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">150 W, hat SS1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HP5–HP8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">150 W, hat SS2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HP9–HP12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">150 W, hat SS3</t>
+  </si>
+  <si>
     <t xml:space="preserve">JB1</t>
   </si>
   <si>
@@ -1316,6 +1337,21 @@
   </si>
   <si>
     <t xml:space="preserve">W16: NYY 3x2,5 mm², L=67 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hoparlör (ses kolu)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W18: NYY 3x2,5 mm², L=100 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kol gücü hoparlörlere eşit bölünmüştür (varsayım)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W19: NYY 3x2,5 mm², L=100 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W20: NYY 3x2,5 mm², L=100 m</t>
   </si>
   <si>
     <t xml:space="preserve">EK KALEMLER</t>
@@ -3181,7 +3217,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
         <v>45</v>
       </c>
@@ -3229,7 +3265,7 @@
         <v>1.15942028985507</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
         <v>47</v>
       </c>
@@ -5647,7 +5683,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
         <v>162</v>
       </c>
@@ -5727,7 +5763,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
         <v>163</v>
       </c>
@@ -6724,7 +6760,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F83"/>
+  <dimension ref="A1:F86"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
@@ -8093,7 +8129,7 @@
         <v>379</v>
       </c>
       <c r="C72" s="22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D72" s="13" t="s">
         <v>380</v>
@@ -8102,67 +8138,67 @@
         <v>335</v>
       </c>
       <c r="F72" s="22" t="s">
-        <v>381</v>
+        <v>356</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="28" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B73" s="13" t="s">
         <v>379</v>
       </c>
       <c r="C73" s="22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D73" s="13" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="E73" s="22" t="s">
         <v>335</v>
       </c>
       <c r="F73" s="22" t="s">
-        <v>381</v>
+        <v>356</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="28" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="B74" s="13" t="s">
         <v>379</v>
       </c>
       <c r="C74" s="22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D74" s="13" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="E74" s="22" t="s">
         <v>335</v>
       </c>
       <c r="F74" s="22" t="s">
-        <v>381</v>
+        <v>356</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="28" t="s">
+        <v>385</v>
+      </c>
+      <c r="B75" s="13" t="s">
         <v>386</v>
-      </c>
-      <c r="B75" s="13" t="s">
-        <v>387</v>
       </c>
       <c r="C75" s="22" t="n">
         <v>1</v>
       </c>
       <c r="D75" s="13" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="E75" s="22" t="s">
         <v>335</v>
       </c>
       <c r="F75" s="22" t="s">
-        <v>381</v>
+        <v>388</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8170,27 +8206,27 @@
         <v>389</v>
       </c>
       <c r="B76" s="13" t="s">
+        <v>386</v>
+      </c>
+      <c r="C76" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D76" s="13" t="s">
         <v>390</v>
-      </c>
-      <c r="C76" s="22" t="n">
-        <v>6</v>
-      </c>
-      <c r="D76" s="13" t="s">
-        <v>391</v>
       </c>
       <c r="E76" s="22" t="s">
         <v>335</v>
       </c>
       <c r="F76" s="22" t="s">
-        <v>346</v>
+        <v>388</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="28" t="s">
-        <v>155</v>
+        <v>391</v>
       </c>
       <c r="B77" s="13" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="C77" s="22" t="n">
         <v>1</v>
@@ -8202,7 +8238,7 @@
         <v>335</v>
       </c>
       <c r="F77" s="22" t="s">
-        <v>346</v>
+        <v>388</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8210,33 +8246,33 @@
         <v>393</v>
       </c>
       <c r="B78" s="13" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="C78" s="22" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D78" s="13" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="E78" s="22" t="s">
         <v>335</v>
       </c>
       <c r="F78" s="22" t="s">
-        <v>346</v>
+        <v>388</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="28" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B79" s="13" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
       <c r="C79" s="22" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D79" s="13" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="E79" s="22" t="s">
         <v>335</v>
@@ -8247,16 +8283,16 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="28" t="s">
+        <v>155</v>
+      </c>
+      <c r="B80" s="13" t="s">
         <v>397</v>
       </c>
-      <c r="B80" s="13" t="s">
-        <v>390</v>
-      </c>
       <c r="C80" s="22" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D80" s="13" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="E80" s="22" t="s">
         <v>335</v>
@@ -8267,16 +8303,16 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="28" t="s">
-        <v>171</v>
+        <v>400</v>
       </c>
       <c r="B81" s="13" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
       <c r="C81" s="22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D81" s="13" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="E81" s="22" t="s">
         <v>335</v>
@@ -8287,41 +8323,101 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="28" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B82" s="13" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
       <c r="C82" s="22" t="n">
         <v>3</v>
       </c>
       <c r="D82" s="13" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="E82" s="22" t="s">
         <v>335</v>
       </c>
       <c r="F82" s="22" t="s">
-        <v>356</v>
+        <v>346</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B83" s="13" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
       <c r="C83" s="22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D83" s="13" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="E83" s="22" t="s">
         <v>335</v>
       </c>
       <c r="F83" s="22" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="28" t="s">
+        <v>171</v>
+      </c>
+      <c r="B84" s="13" t="s">
+        <v>397</v>
+      </c>
+      <c r="C84" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D84" s="13" t="s">
+        <v>406</v>
+      </c>
+      <c r="E84" s="22" t="s">
+        <v>335</v>
+      </c>
+      <c r="F84" s="22" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="28" t="s">
+        <v>407</v>
+      </c>
+      <c r="B85" s="13" t="s">
+        <v>397</v>
+      </c>
+      <c r="C85" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="D85" s="13" t="s">
+        <v>408</v>
+      </c>
+      <c r="E85" s="22" t="s">
+        <v>335</v>
+      </c>
+      <c r="F85" s="22" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="28" t="s">
+        <v>409</v>
+      </c>
+      <c r="B86" s="13" t="s">
+        <v>397</v>
+      </c>
+      <c r="C86" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D86" s="13" t="s">
+        <v>410</v>
+      </c>
+      <c r="E86" s="22" t="s">
+        <v>335</v>
+      </c>
+      <c r="F86" s="22" t="s">
         <v>346</v>
       </c>
     </row>
@@ -8345,7 +8441,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
@@ -8361,7 +8457,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8371,7 +8467,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>405</v>
+        <v>412</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="4" t="n">
@@ -8383,28 +8479,28 @@
         <v>10</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>406</v>
+        <v>413</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>183</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>407</v>
+        <v>414</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>409</v>
+        <v>416</v>
       </c>
       <c r="G5" s="7" t="s">
         <v>13</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>410</v>
+        <v>417</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>411</v>
+        <v>418</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8431,10 +8527,10 @@
         <v>17</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>412</v>
+        <v>419</v>
       </c>
       <c r="I6" s="13" t="s">
-        <v>413</v>
+        <v>420</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8442,7 +8538,7 @@
         <v>357</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="C7" s="10" t="n">
         <v>10</v>
@@ -8461,10 +8557,10 @@
         <v>18</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>415</v>
+        <v>422</v>
       </c>
       <c r="I7" s="13" t="s">
-        <v>416</v>
+        <v>423</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8472,7 +8568,7 @@
         <v>360</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="C8" s="10" t="n">
         <v>10</v>
@@ -8491,10 +8587,10 @@
         <v>19</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>417</v>
+        <v>424</v>
       </c>
       <c r="I8" s="13" t="s">
-        <v>416</v>
+        <v>423</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8502,7 +8598,7 @@
         <v>362</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="C9" s="10" t="n">
         <v>10</v>
@@ -8521,10 +8617,10 @@
         <v>17</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>418</v>
+        <v>425</v>
       </c>
       <c r="I9" s="13" t="s">
-        <v>416</v>
+        <v>423</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8551,10 +8647,10 @@
         <v>18</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>419</v>
+        <v>426</v>
       </c>
       <c r="I10" s="13" t="s">
-        <v>420</v>
+        <v>427</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8581,10 +8677,10 @@
         <v>17</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>421</v>
+        <v>428</v>
       </c>
       <c r="I11" s="13" t="s">
-        <v>420</v>
+        <v>427</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8611,10 +8707,10 @@
         <v>19</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>422</v>
+        <v>429</v>
       </c>
       <c r="I12" s="13" t="s">
-        <v>420</v>
+        <v>427</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8641,10 +8737,10 @@
         <v>19</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>423</v>
+        <v>430</v>
       </c>
       <c r="I13" s="13" t="s">
-        <v>424</v>
+        <v>431</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8671,10 +8767,10 @@
         <v>18</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>425</v>
+        <v>432</v>
       </c>
       <c r="I14" s="13" t="s">
-        <v>424</v>
+        <v>431</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8701,176 +8797,266 @@
         <v>17</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>426</v>
+        <v>433</v>
       </c>
       <c r="I15" s="13" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="14" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="28" t="s">
+        <v>378</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>434</v>
+      </c>
+      <c r="C16" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D16" s="29" t="n">
+        <v>150</v>
+      </c>
+      <c r="E16" s="30" t="n">
+        <f aca="false">C16*D16</f>
+        <v>600</v>
+      </c>
+      <c r="F16" s="31" t="s">
+        <v>55</v>
+      </c>
+      <c r="G16" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="H16" s="8" t="s">
+        <v>435</v>
+      </c>
+      <c r="I16" s="13" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="28" t="s">
+        <v>381</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>434</v>
+      </c>
+      <c r="C17" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D17" s="29" t="n">
+        <v>150</v>
+      </c>
+      <c r="E17" s="30" t="n">
+        <f aca="false">C17*D17</f>
+        <v>600</v>
+      </c>
+      <c r="F17" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="G17" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="H17" s="8" t="s">
+        <v>437</v>
+      </c>
+      <c r="I17" s="13" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="28" t="s">
+        <v>383</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>434</v>
+      </c>
+      <c r="C18" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D18" s="29" t="n">
+        <v>150</v>
+      </c>
+      <c r="E18" s="30" t="n">
+        <f aca="false">C18*D18</f>
+        <v>600</v>
+      </c>
+      <c r="F18" s="31" t="s">
+        <v>59</v>
+      </c>
+      <c r="G18" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="H18" s="8" t="s">
+        <v>438</v>
+      </c>
+      <c r="I18" s="13" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="B16" s="15"/>
-      <c r="C16" s="32" t="n">
-        <f aca="false">SUM(C6:C15)</f>
-        <v>91</v>
-      </c>
-      <c r="D16" s="15"/>
-      <c r="E16" s="32" t="n">
-        <f aca="false">SUM(E6:E15)</f>
-        <v>12750</v>
-      </c>
-      <c r="F16" s="15"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="15"/>
-      <c r="I16" s="15"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14" t="s">
-        <v>427</v>
-      </c>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
-      <c r="I18" s="14"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
-        <v>378</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>379</v>
-      </c>
-      <c r="C19" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="31" t="s">
-        <v>47</v>
-      </c>
-      <c r="G19" s="22" t="s">
-        <v>19</v>
-      </c>
-      <c r="H19" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="I19" s="8" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
-        <v>382</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>379</v>
-      </c>
-      <c r="C20" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="31" t="s">
-        <v>49</v>
-      </c>
-      <c r="G20" s="22" t="s">
-        <v>18</v>
-      </c>
-      <c r="H20" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="I20" s="8" t="s">
-        <v>428</v>
-      </c>
+      <c r="B19" s="15"/>
+      <c r="C19" s="32" t="n">
+        <f aca="false">SUM(C6:C18)</f>
+        <v>103</v>
+      </c>
+      <c r="D19" s="15"/>
+      <c r="E19" s="32" t="n">
+        <f aca="false">SUM(E6:E18)</f>
+        <v>14550</v>
+      </c>
+      <c r="F19" s="15"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="15"/>
+      <c r="I19" s="15"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
-        <v>384</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>379</v>
-      </c>
-      <c r="C21" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="31" t="s">
-        <v>51</v>
-      </c>
-      <c r="G21" s="22" t="s">
-        <v>17</v>
-      </c>
-      <c r="H21" s="8" t="s">
-        <v>170</v>
-      </c>
-      <c r="I21" s="8" t="s">
-        <v>428</v>
-      </c>
+      <c r="A21" s="14" t="s">
+        <v>439</v>
+      </c>
+      <c r="B21" s="14"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="14"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="14"/>
+      <c r="H21" s="14"/>
+      <c r="I21" s="14"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>397</v>
+        <v>385</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>429</v>
-      </c>
-      <c r="C22" s="33" t="n">
+        <v>386</v>
+      </c>
+      <c r="C22" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="31" t="s">
+        <v>47</v>
+      </c>
+      <c r="G22" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="H22" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="I22" s="8" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="C23" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="31" t="s">
+        <v>49</v>
+      </c>
+      <c r="G23" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="H23" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="I23" s="8" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="C24" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="31" t="s">
+        <v>51</v>
+      </c>
+      <c r="G24" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="H24" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="I24" s="8" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>441</v>
+      </c>
+      <c r="C25" s="33" t="n">
         <f aca="false">ROUNDUP(('Kablo Çizelgesi'!K29+'Kablo Çizelgesi'!K30+'Kablo Çizelgesi'!K31)*(1+$C$3/100),0)</f>
         <v>220</v>
       </c>
-      <c r="D22" s="22" t="s">
-        <v>430</v>
-      </c>
-      <c r="E22" s="8"/>
-      <c r="F22" s="22" t="s">
-        <v>431</v>
-      </c>
-      <c r="G22" s="22" t="s">
+      <c r="D25" s="22" t="s">
+        <v>442</v>
+      </c>
+      <c r="E25" s="8"/>
+      <c r="F25" s="22" t="s">
+        <v>443</v>
+      </c>
+      <c r="G25" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="H22" s="8" t="s">
-        <v>432</v>
-      </c>
-      <c r="I22" s="8" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="s">
-        <v>386</v>
-      </c>
-      <c r="B23" s="8" t="s">
-        <v>434</v>
-      </c>
-      <c r="C23" s="10" t="n">
+      <c r="H25" s="8" t="s">
+        <v>444</v>
+      </c>
+      <c r="I25" s="8" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>446</v>
+      </c>
+      <c r="C26" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22" t="s">
+      <c r="D26" s="22"/>
+      <c r="E26" s="22"/>
+      <c r="F26" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="G23" s="22" t="s">
+      <c r="G26" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="H23" s="8" t="s">
-        <v>435</v>
-      </c>
-      <c r="I23" s="8" t="s">
-        <v>436</v>
+      <c r="H26" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="I26" s="8" t="s">
+        <v>448</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A18:I18"/>
+    <mergeCell ref="A21:I21"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -8900,7 +9086,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>437</v>
+        <v>449</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8910,7 +9096,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>438</v>
+        <v>450</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="4" t="n">
@@ -8919,7 +9105,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>439</v>
+        <v>451</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="4" t="n">
@@ -8928,7 +9114,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>440</v>
+        <v>452</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="4" t="n">
@@ -8937,7 +9123,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>441</v>
+        <v>453</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="4" t="n">
@@ -8946,7 +9132,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>442</v>
+        <v>454</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="4" t="n">
@@ -8955,7 +9141,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>443</v>
+        <v>455</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="4" t="n">
@@ -8964,7 +9150,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>444</v>
+        <v>456</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="4" t="n">
@@ -8973,7 +9159,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>445</v>
+        <v>457</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="4" t="n">
@@ -8982,7 +9168,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>446</v>
+        <v>458</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="4" t="n">
@@ -8991,7 +9177,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>447</v>
+        <v>459</v>
       </c>
       <c r="B12" s="3"/>
       <c r="C12" s="4" t="n">
@@ -9000,7 +9186,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>448</v>
+        <v>460</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="4" t="n">
@@ -9009,7 +9195,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>449</v>
+        <v>461</v>
       </c>
       <c r="B14" s="3"/>
       <c r="C14" s="4" t="n">
@@ -9018,7 +9204,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>450</v>
+        <v>462</v>
       </c>
       <c r="B15" s="3"/>
       <c r="C15" s="4" t="n">
@@ -9027,7 +9213,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>451</v>
+        <v>463</v>
       </c>
       <c r="B16" s="3"/>
       <c r="C16" s="4" t="n">
@@ -9036,7 +9222,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>452</v>
+        <v>464</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="4" t="n">
@@ -9045,7 +9231,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>453</v>
+        <v>465</v>
       </c>
       <c r="B18" s="3"/>
       <c r="C18" s="4" t="n">
@@ -9054,7 +9240,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>454</v>
+        <v>466</v>
       </c>
       <c r="B19" s="3"/>
       <c r="C19" s="4" t="n">
@@ -9063,7 +9249,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>455</v>
+        <v>467</v>
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="4" t="n">
@@ -9072,7 +9258,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>456</v>
+        <v>468</v>
       </c>
       <c r="B21" s="3"/>
       <c r="C21" s="4" t="n">
@@ -9081,7 +9267,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>457</v>
+        <v>469</v>
       </c>
       <c r="B22" s="3"/>
       <c r="C22" s="4" t="n">
@@ -9090,7 +9276,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>458</v>
+        <v>470</v>
       </c>
       <c r="B23" s="3"/>
       <c r="C23" s="4" t="n">
@@ -9099,7 +9285,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>459</v>
+        <v>471</v>
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="4" t="n">
@@ -9108,7 +9294,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>460</v>
+        <v>472</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="4" t="n">
@@ -9120,16 +9306,16 @@
         <v>10</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>461</v>
+        <v>473</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>462</v>
+        <v>474</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>463</v>
+        <v>475</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>464</v>
+        <v>476</v>
       </c>
       <c r="F27" s="6" t="s">
         <v>184</v>
@@ -9137,313 +9323,313 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="28" t="s">
-        <v>465</v>
+        <v>477</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>466</v>
+        <v>478</v>
       </c>
       <c r="C28" s="22" t="s">
-        <v>430</v>
+        <v>442</v>
       </c>
       <c r="D28" s="33" t="n">
         <f aca="false">2*(($C$3+2*$C$5)+($C$4+2*$C$5))</f>
         <v>88</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>467</v>
+        <v>479</v>
       </c>
       <c r="F28" s="13" t="s">
-        <v>468</v>
+        <v>480</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="28" t="s">
-        <v>465</v>
+        <v>477</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>469</v>
+        <v>481</v>
       </c>
       <c r="C29" s="22" t="s">
-        <v>430</v>
+        <v>442</v>
       </c>
       <c r="D29" s="33" t="n">
         <f aca="false">ROUNDUP(D28*(1+$C$10/100),0)</f>
         <v>97</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>470</v>
+        <v>482</v>
       </c>
       <c r="F29" s="13" t="s">
-        <v>468</v>
+        <v>480</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="28" t="s">
-        <v>471</v>
+        <v>483</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>472</v>
+        <v>484</v>
       </c>
       <c r="C30" s="22" t="s">
-        <v>473</v>
+        <v>485</v>
       </c>
       <c r="D30" s="33" t="n">
         <f aca="false">2*(ROUNDUP(($C$3+2*$C$5)/$C$8,0)+ROUNDUP(($C$4+2*$C$5)/$C$8,0))</f>
         <v>12</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>474</v>
+        <v>486</v>
       </c>
       <c r="F30" s="13" t="s">
-        <v>475</v>
+        <v>487</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="28" t="s">
-        <v>471</v>
+        <v>483</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>476</v>
+        <v>488</v>
       </c>
       <c r="C31" s="22" t="s">
-        <v>430</v>
+        <v>442</v>
       </c>
       <c r="D31" s="33" t="n">
         <f aca="false">D30*$C$7</f>
         <v>36</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="F31" s="13"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="28" t="s">
-        <v>471</v>
+        <v>483</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>478</v>
+        <v>490</v>
       </c>
       <c r="C32" s="22" t="s">
-        <v>430</v>
+        <v>442</v>
       </c>
       <c r="D32" s="18" t="n">
         <f aca="false">MAX(($C$3+2*$C$5)/ROUNDUP(($C$3+2*$C$5)/$C$8,0),($C$4+2*$C$5)/ROUNDUP(($C$4+2*$C$5)/$C$8,0))</f>
         <v>7.33333333333333</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>479</v>
+        <v>491</v>
       </c>
       <c r="F32" s="13" t="s">
-        <v>480</v>
+        <v>492</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="28" t="s">
-        <v>481</v>
+        <v>493</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>482</v>
+        <v>494</v>
       </c>
       <c r="C33" s="22" t="s">
-        <v>473</v>
+        <v>485</v>
       </c>
       <c r="D33" s="33" t="n">
         <f aca="false">$C$15</f>
         <v>4</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>483</v>
+        <v>495</v>
       </c>
       <c r="F33" s="13" t="s">
-        <v>484</v>
+        <v>496</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="28" t="s">
+        <v>497</v>
+      </c>
+      <c r="B34" s="13" t="s">
+        <v>498</v>
+      </c>
+      <c r="C34" s="22" t="s">
         <v>485</v>
-      </c>
-      <c r="B34" s="13" t="s">
-        <v>486</v>
-      </c>
-      <c r="C34" s="22" t="s">
-        <v>473</v>
       </c>
       <c r="D34" s="33" t="n">
         <f aca="false">MIN(8,MAX(2,ROUNDUP(2*($C$3+$C$4)/$C$9,0)))</f>
         <v>6</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>487</v>
+        <v>499</v>
       </c>
       <c r="F34" s="13" t="s">
-        <v>488</v>
+        <v>500</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="28" t="s">
-        <v>489</v>
+        <v>501</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>490</v>
+        <v>502</v>
       </c>
       <c r="C35" s="22" t="s">
-        <v>473</v>
+        <v>485</v>
       </c>
       <c r="D35" s="33" t="n">
         <f aca="false">D34</f>
         <v>6</v>
       </c>
       <c r="E35" s="13" t="s">
-        <v>491</v>
+        <v>503</v>
       </c>
       <c r="F35" s="13" t="s">
-        <v>492</v>
+        <v>504</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="28" t="s">
-        <v>485</v>
+        <v>497</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>493</v>
+        <v>505</v>
       </c>
       <c r="C36" s="22" t="s">
-        <v>430</v>
+        <v>442</v>
       </c>
       <c r="D36" s="33" t="n">
         <f aca="false">ROUNDUP((D34*($C$11+$C$6)+($C$13-$C$11)+(PI()*$C$14/2+2))*(1+$C$10/100),0)</f>
         <v>101</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>494</v>
+        <v>506</v>
       </c>
       <c r="F36" s="13" t="s">
-        <v>495</v>
+        <v>507</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="28" t="s">
-        <v>496</v>
+        <v>508</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>497</v>
+        <v>509</v>
       </c>
       <c r="C37" s="22" t="s">
-        <v>430</v>
+        <v>442</v>
       </c>
       <c r="D37" s="33" t="n">
         <f aca="false">ROUNDUP((2*($C$3+$C$4)+$C$4/2+3)*(1+$C$10/100),0)</f>
         <v>103</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>498</v>
+        <v>510</v>
       </c>
       <c r="F37" s="13" t="s">
-        <v>499</v>
+        <v>511</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="28" t="s">
-        <v>500</v>
+        <v>512</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>501</v>
+        <v>513</v>
       </c>
       <c r="C38" s="22" t="s">
-        <v>473</v>
+        <v>485</v>
       </c>
       <c r="D38" s="33" t="n">
         <f aca="false">3</f>
         <v>3</v>
       </c>
       <c r="E38" s="13" t="s">
-        <v>502</v>
+        <v>514</v>
       </c>
       <c r="F38" s="13" t="s">
-        <v>503</v>
+        <v>515</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="28" t="s">
-        <v>500</v>
+        <v>512</v>
       </c>
       <c r="B39" s="13" t="s">
-        <v>504</v>
+        <v>516</v>
       </c>
       <c r="C39" s="22" t="s">
-        <v>430</v>
+        <v>442</v>
       </c>
       <c r="D39" s="20" t="n">
         <f aca="false">$C$23+$C$24+$C$25</f>
         <v>4.5</v>
       </c>
       <c r="E39" s="13" t="s">
-        <v>505</v>
+        <v>517</v>
       </c>
       <c r="F39" s="13"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="28" t="s">
-        <v>506</v>
+        <v>518</v>
       </c>
       <c r="B40" s="13" t="s">
-        <v>507</v>
+        <v>519</v>
       </c>
       <c r="C40" s="22" t="s">
-        <v>473</v>
+        <v>485</v>
       </c>
       <c r="D40" s="33" t="n">
         <f aca="false">1</f>
         <v>1</v>
       </c>
       <c r="E40" s="13" t="s">
-        <v>508</v>
+        <v>520</v>
       </c>
       <c r="F40" s="13" t="s">
-        <v>509</v>
+        <v>521</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="28" t="s">
-        <v>510</v>
+        <v>522</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>511</v>
+        <v>523</v>
       </c>
       <c r="C41" s="22" t="s">
-        <v>430</v>
+        <v>442</v>
       </c>
       <c r="D41" s="33" t="n">
         <f aca="false">ROUNDUP($C$16*(1+$C$10/100),0)</f>
         <v>3</v>
       </c>
       <c r="E41" s="13" t="s">
-        <v>512</v>
+        <v>524</v>
       </c>
       <c r="F41" s="13" t="s">
-        <v>495</v>
+        <v>507</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="28" t="s">
-        <v>513</v>
+        <v>525</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>514</v>
+        <v>526</v>
       </c>
       <c r="C42" s="22" t="s">
-        <v>430</v>
+        <v>442</v>
       </c>
       <c r="D42" s="33" t="n">
         <f aca="false">ROUNDUP($C$17*(1+$C$10/100),0)</f>
         <v>4</v>
       </c>
       <c r="E42" s="13" t="s">
-        <v>512</v>
+        <v>524</v>
       </c>
       <c r="F42" s="13" t="s">
-        <v>495</v>
+        <v>507</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9451,167 +9637,167 @@
         <v>340</v>
       </c>
       <c r="B43" s="13" t="s">
-        <v>515</v>
+        <v>527</v>
       </c>
       <c r="C43" s="22" t="s">
-        <v>430</v>
+        <v>442</v>
       </c>
       <c r="D43" s="33" t="n">
         <f aca="false">ROUNDUP($C$22*(1+$C$10/100),0)</f>
         <v>33</v>
       </c>
       <c r="E43" s="13" t="s">
-        <v>516</v>
+        <v>528</v>
       </c>
       <c r="F43" s="13" t="s">
-        <v>517</v>
+        <v>529</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="28" t="s">
-        <v>518</v>
+        <v>530</v>
       </c>
       <c r="B44" s="13" t="s">
-        <v>519</v>
+        <v>531</v>
       </c>
       <c r="C44" s="22" t="s">
-        <v>473</v>
+        <v>485</v>
       </c>
       <c r="D44" s="33" t="n">
         <f aca="false">$C$18</f>
         <v>3</v>
       </c>
       <c r="E44" s="13" t="s">
-        <v>483</v>
+        <v>495</v>
       </c>
       <c r="F44" s="13" t="s">
-        <v>520</v>
+        <v>532</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="28" t="s">
-        <v>518</v>
+        <v>530</v>
       </c>
       <c r="B45" s="13" t="s">
-        <v>521</v>
+        <v>533</v>
       </c>
       <c r="C45" s="22" t="s">
-        <v>430</v>
+        <v>442</v>
       </c>
       <c r="D45" s="33" t="n">
         <f aca="false">($C$18-1)*$C$19+6</f>
         <v>18</v>
       </c>
       <c r="E45" s="13" t="s">
-        <v>522</v>
+        <v>534</v>
       </c>
       <c r="F45" s="13" t="s">
-        <v>523</v>
+        <v>535</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="28" t="s">
-        <v>524</v>
+        <v>536</v>
       </c>
       <c r="B46" s="13" t="s">
-        <v>525</v>
+        <v>537</v>
       </c>
       <c r="C46" s="22" t="s">
-        <v>430</v>
+        <v>442</v>
       </c>
       <c r="D46" s="33" t="n">
         <f aca="false">ROUNDUP($C$21*$C$20*(1+$C$10/100),0)</f>
         <v>80</v>
       </c>
       <c r="E46" s="13" t="s">
-        <v>526</v>
+        <v>538</v>
       </c>
       <c r="F46" s="13" t="s">
-        <v>527</v>
+        <v>539</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="28" t="s">
-        <v>524</v>
+        <v>536</v>
       </c>
       <c r="B47" s="13" t="s">
-        <v>528</v>
+        <v>540</v>
       </c>
       <c r="C47" s="22" t="s">
-        <v>473</v>
+        <v>485</v>
       </c>
       <c r="D47" s="33" t="n">
         <f aca="false">$C$21</f>
         <v>6</v>
       </c>
       <c r="E47" s="13" t="s">
-        <v>529</v>
+        <v>541</v>
       </c>
       <c r="F47" s="13" t="s">
-        <v>530</v>
+        <v>542</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="28" t="s">
-        <v>531</v>
+        <v>543</v>
       </c>
       <c r="B48" s="13" t="s">
-        <v>532</v>
+        <v>544</v>
       </c>
       <c r="C48" s="22" t="s">
-        <v>473</v>
+        <v>485</v>
       </c>
       <c r="D48" s="33" t="n">
         <f aca="false">1</f>
         <v>1</v>
       </c>
       <c r="E48" s="13" t="s">
-        <v>533</v>
+        <v>545</v>
       </c>
       <c r="F48" s="13" t="s">
-        <v>534</v>
+        <v>546</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="28" t="s">
-        <v>535</v>
+        <v>547</v>
       </c>
       <c r="B49" s="13" t="s">
-        <v>536</v>
+        <v>548</v>
       </c>
       <c r="C49" s="22" t="s">
-        <v>473</v>
+        <v>485</v>
       </c>
       <c r="D49" s="33" t="n">
         <f aca="false">D30+D34+2+1+$C$21</f>
         <v>27</v>
       </c>
       <c r="E49" s="13" t="s">
-        <v>537</v>
+        <v>549</v>
       </c>
       <c r="F49" s="13" t="s">
-        <v>538</v>
+        <v>550</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="28" t="s">
-        <v>535</v>
+        <v>547</v>
       </c>
       <c r="B50" s="13" t="s">
-        <v>539</v>
+        <v>551</v>
       </c>
       <c r="C50" s="22" t="s">
-        <v>473</v>
+        <v>485</v>
       </c>
       <c r="D50" s="33" t="n">
         <f aca="false">3</f>
         <v>3</v>
       </c>
       <c r="E50" s="13" t="s">
-        <v>540</v>
+        <v>552</v>
       </c>
       <c r="F50" s="13" t="s">
-        <v>541</v>
+        <v>553</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9619,17 +9805,17 @@
         <v>67</v>
       </c>
       <c r="B51" s="13" t="s">
-        <v>542</v>
+        <v>554</v>
       </c>
       <c r="C51" s="22" t="s">
-        <v>473</v>
+        <v>485</v>
       </c>
       <c r="D51" s="33" t="n">
         <f aca="false">ROUNDUP(D49/10,0)</f>
         <v>3</v>
       </c>
       <c r="E51" s="13" t="s">
-        <v>543</v>
+        <v>555</v>
       </c>
       <c r="F51" s="13"/>
     </row>
@@ -9691,7 +9877,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>544</v>
+        <v>556</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9701,7 +9887,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>545</v>
+        <v>557</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -9721,7 +9907,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>546</v>
+        <v>558</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -9731,7 +9917,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>547</v>
+        <v>559</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -9741,7 +9927,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>548</v>
+        <v>560</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
@@ -9751,7 +9937,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>549</v>
+        <v>561</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -9771,7 +9957,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>550</v>
+        <v>562</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -9781,7 +9967,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>551</v>
+        <v>563</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -9801,7 +9987,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>552</v>
+        <v>564</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -9811,7 +9997,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>553</v>
+        <v>565</v>
       </c>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -9821,7 +10007,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>554</v>
+        <v>566</v>
       </c>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -9831,7 +10017,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>555</v>
+        <v>567</v>
       </c>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -9841,7 +10027,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>556</v>
+        <v>568</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -9851,7 +10037,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>557</v>
+        <v>569</v>
       </c>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -9861,7 +10047,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>558</v>
+        <v>570</v>
       </c>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -9871,7 +10057,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>559</v>
+        <v>571</v>
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -9881,7 +10067,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="14" t="s">
-        <v>560</v>
+        <v>572</v>
       </c>
       <c r="B22" s="14"/>
       <c r="C22" s="14"/>
@@ -9895,7 +10081,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>561</v>
+        <v>573</v>
       </c>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -9904,12 +10090,12 @@
         <v>360.843918243516</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>562</v>
+        <v>574</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>563</v>
+        <v>575</v>
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -9918,12 +10104,12 @@
         <v>9.0210979560879</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>564</v>
+        <v>576</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>565</v>
+        <v>577</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -9932,12 +10118,12 @@
         <v>0.0256</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>566</v>
+        <v>578</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>567</v>
+        <v>579</v>
       </c>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
@@ -9946,12 +10132,12 @@
         <v>0.00832</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>566</v>
+        <v>578</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>568</v>
+        <v>580</v>
       </c>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
@@ -9960,12 +10146,12 @@
         <v>0.0242102788088035</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>566</v>
+        <v>578</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>569</v>
+        <v>581</v>
       </c>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
@@ -9974,12 +10160,12 @@
         <v>0.0056390977443609</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>566</v>
+        <v>578</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>570</v>
+        <v>582</v>
       </c>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -9988,12 +10174,12 @@
         <v>0.0024</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>566</v>
+        <v>578</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>571</v>
+        <v>583</v>
       </c>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
@@ -10002,12 +10188,12 @@
         <v>0.0300493485473292</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>566</v>
+        <v>578</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>572</v>
+        <v>584</v>
       </c>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
@@ -10016,12 +10202,12 @@
         <v>7.68536154160241</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>564</v>
+        <v>576</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="s">
-        <v>573</v>
+        <v>585</v>
       </c>
       <c r="B33" s="14"/>
       <c r="C33" s="14"/>
@@ -10035,45 +10221,45 @@
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>574</v>
+        <v>586</v>
       </c>
       <c r="B34" s="7" t="s">
         <v>10</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>575</v>
+        <v>587</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>576</v>
+        <v>588</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>577</v>
+        <v>589</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>578</v>
+        <v>590</v>
       </c>
       <c r="G34" s="7" t="s">
-        <v>579</v>
+        <v>591</v>
       </c>
       <c r="H34" s="7" t="s">
-        <v>580</v>
+        <v>592</v>
       </c>
       <c r="I34" s="7" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="J34" s="7" t="s">
-        <v>411</v>
+        <v>418</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="22" t="s">
-        <v>582</v>
+        <v>594</v>
       </c>
       <c r="B35" s="28" t="s">
         <v>141</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>583</v>
+        <v>595</v>
       </c>
       <c r="D35" s="22" t="n">
         <f aca="false">$D$12</f>
@@ -10099,18 +10285,18 @@
         <v>UYGUN</v>
       </c>
       <c r="J35" s="13" t="s">
-        <v>584</v>
+        <v>596</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="22" t="s">
-        <v>585</v>
+        <v>597</v>
       </c>
       <c r="B36" s="28" t="s">
         <v>199</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>586</v>
+        <v>598</v>
       </c>
       <c r="D36" s="22" t="s">
         <v>67</v>
@@ -10136,18 +10322,18 @@
         <v>UYGUN</v>
       </c>
       <c r="J36" s="13" t="s">
-        <v>587</v>
+        <v>599</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="22" t="s">
-        <v>588</v>
+        <v>600</v>
       </c>
       <c r="B37" s="28" t="s">
         <v>273</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>589</v>
+        <v>601</v>
       </c>
       <c r="D37" s="22" t="n">
         <v>63</v>
@@ -10171,18 +10357,18 @@
         <v>UYGUN</v>
       </c>
       <c r="J37" s="13" t="s">
-        <v>590</v>
+        <v>602</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="22" t="s">
-        <v>588</v>
+        <v>600</v>
       </c>
       <c r="B38" s="28" t="s">
         <v>240</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>591</v>
+        <v>603</v>
       </c>
       <c r="D38" s="22" t="n">
         <v>25</v>
@@ -10206,18 +10392,18 @@
         <v>UYGUN</v>
       </c>
       <c r="J38" s="13" t="s">
-        <v>592</v>
+        <v>604</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="22" t="s">
-        <v>588</v>
+        <v>600</v>
       </c>
       <c r="B39" s="28" t="s">
         <v>243</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>593</v>
+        <v>605</v>
       </c>
       <c r="D39" s="22" t="n">
         <v>25</v>
@@ -10240,18 +10426,18 @@
         <v>UYGUN</v>
       </c>
       <c r="J39" s="13" t="s">
-        <v>594</v>
+        <v>606</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="22" t="s">
-        <v>588</v>
+        <v>600</v>
       </c>
       <c r="B40" s="28" t="s">
         <v>276</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>595</v>
+        <v>607</v>
       </c>
       <c r="D40" s="22" t="n">
         <v>63</v>
@@ -10274,18 +10460,18 @@
         <v>UYGUN</v>
       </c>
       <c r="J40" s="13" t="s">
-        <v>596</v>
+        <v>608</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="22" t="s">
-        <v>597</v>
+        <v>609</v>
       </c>
       <c r="B41" s="28" t="s">
         <v>279</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>598</v>
+        <v>610</v>
       </c>
       <c r="D41" s="22" t="n">
         <v>14</v>
@@ -10312,16 +10498,16 @@
     </row>
     <row r="42" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="22" t="s">
-        <v>597</v>
+        <v>609</v>
       </c>
       <c r="B42" s="28" t="s">
-        <v>599</v>
+        <v>611</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>600</v>
+        <v>612</v>
       </c>
       <c r="D42" s="22" t="s">
-        <v>601</v>
+        <v>613</v>
       </c>
       <c r="E42" s="22" t="n">
         <v>30</v>
@@ -10341,18 +10527,18 @@
         <v>UYGUN</v>
       </c>
       <c r="J42" s="13" t="s">
-        <v>602</v>
+        <v>614</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="22" t="s">
-        <v>597</v>
+        <v>609</v>
       </c>
       <c r="B43" s="28" t="s">
         <v>282</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>603</v>
+        <v>615</v>
       </c>
       <c r="D43" s="22" t="n">
         <v>25</v>
@@ -10375,18 +10561,18 @@
         <v>UYGUN</v>
       </c>
       <c r="J43" s="13" t="s">
-        <v>604</v>
+        <v>616</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="22" t="s">
-        <v>605</v>
+        <v>617</v>
       </c>
       <c r="B44" s="28" t="s">
         <v>297</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>606</v>
+        <v>618</v>
       </c>
       <c r="D44" s="22" t="n">
         <v>10</v>
@@ -10410,15 +10596,15 @@
         <v>UYGUN</v>
       </c>
       <c r="J44" s="13" t="s">
-        <v>607</v>
+        <v>619</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="3" t="s">
-        <v>608</v>
+        <v>620</v>
       </c>
       <c r="C45" s="8" t="s">
-        <v>609</v>
+        <v>621</v>
       </c>
       <c r="G45" s="8" t="n">
         <f aca="false">$D$10</f>
@@ -10435,7 +10621,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="14" t="s">
-        <v>610</v>
+        <v>622</v>
       </c>
       <c r="B47" s="14"/>
       <c r="C47" s="14"/>
@@ -10449,34 +10635,34 @@
     </row>
     <row r="48" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
-        <v>611</v>
+        <v>623</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>612</v>
+        <v>624</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>613</v>
+        <v>625</v>
       </c>
       <c r="D48" s="7" t="s">
-        <v>614</v>
+        <v>626</v>
       </c>
       <c r="E48" s="7" t="s">
-        <v>615</v>
+        <v>627</v>
       </c>
       <c r="F48" s="7" t="s">
-        <v>616</v>
+        <v>628</v>
       </c>
       <c r="G48" s="7" t="s">
-        <v>617</v>
+        <v>629</v>
       </c>
       <c r="H48" s="7" t="s">
-        <v>618</v>
+        <v>630</v>
       </c>
       <c r="I48" s="7" t="s">
-        <v>619</v>
+        <v>631</v>
       </c>
       <c r="J48" s="7" t="s">
-        <v>620</v>
+        <v>632</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10484,7 +10670,7 @@
         <v>199</v>
       </c>
       <c r="B49" s="13" t="s">
-        <v>621</v>
+        <v>633</v>
       </c>
       <c r="C49" s="8" t="n">
         <f aca="false">$D$15</f>
@@ -10522,7 +10708,7 @@
         <v>199</v>
       </c>
       <c r="B50" s="13" t="s">
-        <v>622</v>
+        <v>634</v>
       </c>
       <c r="C50" s="8" t="n">
         <f aca="false">$D$15</f>
@@ -10560,7 +10746,7 @@
         <v>199</v>
       </c>
       <c r="B51" s="13" t="s">
-        <v>623</v>
+        <v>635</v>
       </c>
       <c r="C51" s="8" t="n">
         <f aca="false">$D$15</f>
@@ -10595,7 +10781,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="14" t="s">
-        <v>624</v>
+        <v>636</v>
       </c>
       <c r="B53" s="14"/>
       <c r="C53" s="14"/>
@@ -10609,29 +10795,29 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="6" t="s">
-        <v>625</v>
+        <v>637</v>
       </c>
       <c r="B54" s="6"/>
       <c r="C54" s="6"/>
       <c r="D54" s="6" t="s">
-        <v>626</v>
+        <v>638</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>462</v>
+        <v>474</v>
       </c>
       <c r="F54" s="6" t="s">
-        <v>627</v>
+        <v>639</v>
       </c>
       <c r="G54" s="6"/>
       <c r="H54" s="6"/>
       <c r="I54" s="6"/>
       <c r="J54" s="6" t="s">
-        <v>411</v>
+        <v>418</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>628</v>
+        <v>640</v>
       </c>
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
@@ -10640,15 +10826,15 @@
         <v>960</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>562</v>
+        <v>574</v>
       </c>
       <c r="J55" s="13" t="s">
-        <v>629</v>
+        <v>641</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>630</v>
+        <v>642</v>
       </c>
       <c r="B56" s="3"/>
       <c r="C56" s="3"/>
@@ -10657,19 +10843,19 @@
         <v>100</v>
       </c>
       <c r="E56" s="8" t="s">
-        <v>631</v>
+        <v>643</v>
       </c>
       <c r="F56" s="24" t="str">
         <f aca="false">IF(D56&gt;=$D$19+$D$18,"UYGUN","UYGUN DEĞİL")</f>
         <v>UYGUN</v>
       </c>
       <c r="J56" s="13" t="s">
-        <v>632</v>
+        <v>644</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
-        <v>633</v>
+        <v>645</v>
       </c>
       <c r="B57" s="3"/>
       <c r="C57" s="3"/>
@@ -10678,19 +10864,19 @@
         <v>10</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>564</v>
+        <v>576</v>
       </c>
       <c r="F57" s="24" t="str">
         <f aca="false">IF(D57&gt;=$D$31,"UYGUN","UYGUN DEĞİL")</f>
         <v>UYGUN</v>
       </c>
       <c r="J57" s="13" t="s">
-        <v>634</v>
+        <v>646</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>635</v>
+        <v>647</v>
       </c>
       <c r="B58" s="3"/>
       <c r="C58" s="3"/>
@@ -10699,20 +10885,20 @@
         <v>7.68536154160241</v>
       </c>
       <c r="E58" s="8" t="s">
-        <v>564</v>
+        <v>576</v>
       </c>
       <c r="J58" s="13" t="s">
-        <v>636</v>
+        <v>648</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="25" t="s">
-        <v>637</v>
+        <v>649</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="25" t="s">
-        <v>638</v>
+        <v>650</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Çizim 6: ses amfisi yeri (AMF1) elektrik odasına eklendi, poz kaydı ve malzeme listesine işlendi
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NjS5sn9fPFLq7X5eqGJ5mC
</commit_message>
<xml_diff>
--- a/cikti/04_hesap_tablolari.xlsx
+++ b/cikti/04_hesap_tablolari.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1227" uniqueCount="651">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1232" uniqueCount="654">
   <si>
     <t xml:space="preserve">YÜK DENGESİ VE FAZ DENGESİZLİĞİ</t>
   </si>
@@ -1078,6 +1078,18 @@
     <t xml:space="preserve">Ç1</t>
   </si>
   <si>
+    <t xml:space="preserve">AMF1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ses amfisi (çok bölgeli, raf tipi)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,8 kW toplam ses hattı gücü; elektrik odasında PN1 yanı (yer varsayımı)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ç6</t>
+  </si>
+  <si>
     <t xml:space="preserve">UPS1</t>
   </si>
   <si>
@@ -1199,9 +1211,6 @@
   </si>
   <si>
     <t xml:space="preserve">hat PJ1, IP65, 3x2,5 mm² geçişli</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ç6</t>
   </si>
   <si>
     <t xml:space="preserve">JB2</t>
@@ -6760,7 +6769,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F86"/>
+  <dimension ref="A1:F87"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
@@ -7898,21 +7907,21 @@
         <v>335</v>
       </c>
       <c r="F60" s="22" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="28" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B61" s="13" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C61" s="22" t="n">
         <v>1</v>
       </c>
       <c r="D61" s="13" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E61" s="22" t="s">
         <v>335</v>
@@ -7921,24 +7930,24 @@
         <v>346</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="28" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B62" s="13" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C62" s="22" t="n">
         <v>1</v>
       </c>
       <c r="D62" s="13" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="E62" s="22" t="s">
         <v>335</v>
       </c>
       <c r="F62" s="22" t="s">
-        <v>356</v>
+        <v>346</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7949,7 +7958,7 @@
         <v>358</v>
       </c>
       <c r="C63" s="22" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D63" s="13" t="s">
         <v>359</v>
@@ -7958,247 +7967,247 @@
         <v>335</v>
       </c>
       <c r="F63" s="22" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="28" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B64" s="13" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="C64" s="22" t="n">
         <v>10</v>
       </c>
       <c r="D64" s="13" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="E64" s="22" t="s">
         <v>335</v>
       </c>
       <c r="F64" s="22" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="28" t="s">
+        <v>364</v>
+      </c>
+      <c r="B65" s="13" t="s">
         <v>362</v>
-      </c>
-      <c r="B65" s="13" t="s">
-        <v>358</v>
       </c>
       <c r="C65" s="22" t="n">
         <v>10</v>
       </c>
       <c r="D65" s="13" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="E65" s="22" t="s">
         <v>335</v>
       </c>
       <c r="F65" s="22" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="28" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B66" s="13" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="C66" s="22" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="D66" s="13" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E66" s="22" t="s">
         <v>335</v>
       </c>
       <c r="F66" s="22" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="28" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B67" s="13" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="C67" s="22" t="n">
         <v>17</v>
       </c>
       <c r="D67" s="13" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="E67" s="22" t="s">
         <v>335</v>
       </c>
       <c r="F67" s="22" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="28" t="s">
+        <v>371</v>
+      </c>
+      <c r="B68" s="13" t="s">
         <v>369</v>
       </c>
-      <c r="B68" s="13" t="s">
-        <v>365</v>
-      </c>
       <c r="C68" s="22" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D68" s="13" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="E68" s="22" t="s">
         <v>335</v>
       </c>
       <c r="F68" s="22" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="28" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B69" s="13" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="C69" s="22" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="D69" s="13" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="E69" s="22" t="s">
         <v>335</v>
       </c>
       <c r="F69" s="22" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="28" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B70" s="13" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="C70" s="22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D70" s="13" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="E70" s="22" t="s">
         <v>335</v>
       </c>
       <c r="F70" s="22" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="28" t="s">
+        <v>378</v>
+      </c>
+      <c r="B71" s="13" t="s">
         <v>376</v>
-      </c>
-      <c r="B71" s="13" t="s">
-        <v>372</v>
       </c>
       <c r="C71" s="22" t="n">
         <v>3</v>
       </c>
       <c r="D71" s="13" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="E71" s="22" t="s">
         <v>335</v>
       </c>
       <c r="F71" s="22" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="28" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B72" s="13" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="C72" s="22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D72" s="13" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="E72" s="22" t="s">
         <v>335</v>
       </c>
       <c r="F72" s="22" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="28" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B73" s="13" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="C73" s="22" t="n">
         <v>4</v>
       </c>
       <c r="D73" s="13" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="E73" s="22" t="s">
         <v>335</v>
       </c>
       <c r="F73" s="22" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="28" t="s">
+        <v>385</v>
+      </c>
+      <c r="B74" s="13" t="s">
         <v>383</v>
-      </c>
-      <c r="B74" s="13" t="s">
-        <v>379</v>
       </c>
       <c r="C74" s="22" t="n">
         <v>4</v>
       </c>
       <c r="D74" s="13" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="E74" s="22" t="s">
         <v>335</v>
       </c>
       <c r="F74" s="22" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="28" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B75" s="13" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="C75" s="22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D75" s="13" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="E75" s="22" t="s">
         <v>335</v>
       </c>
       <c r="F75" s="22" t="s">
-        <v>388</v>
+        <v>360</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8206,47 +8215,47 @@
         <v>389</v>
       </c>
       <c r="B76" s="13" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="C76" s="22" t="n">
         <v>1</v>
       </c>
       <c r="D76" s="13" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="E76" s="22" t="s">
         <v>335</v>
       </c>
       <c r="F76" s="22" t="s">
-        <v>388</v>
+        <v>350</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="28" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B77" s="13" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="C77" s="22" t="n">
         <v>1</v>
       </c>
       <c r="D77" s="13" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="E77" s="22" t="s">
         <v>335</v>
       </c>
       <c r="F77" s="22" t="s">
-        <v>388</v>
+        <v>350</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="28" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B78" s="13" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="C78" s="22" t="n">
         <v>1</v>
@@ -8258,7 +8267,7 @@
         <v>335</v>
       </c>
       <c r="F78" s="22" t="s">
-        <v>388</v>
+        <v>350</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8269,7 +8278,7 @@
         <v>397</v>
       </c>
       <c r="C79" s="22" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D79" s="13" t="s">
         <v>398</v>
@@ -8278,21 +8287,21 @@
         <v>335</v>
       </c>
       <c r="F79" s="22" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="28" t="s">
-        <v>155</v>
+        <v>399</v>
       </c>
       <c r="B80" s="13" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="C80" s="22" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D80" s="13" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="E80" s="22" t="s">
         <v>335</v>
@@ -8303,16 +8312,16 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="28" t="s">
+        <v>155</v>
+      </c>
+      <c r="B81" s="13" t="s">
         <v>400</v>
       </c>
-      <c r="B81" s="13" t="s">
-        <v>397</v>
-      </c>
       <c r="C81" s="22" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D81" s="13" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E81" s="22" t="s">
         <v>335</v>
@@ -8323,16 +8332,16 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="28" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B82" s="13" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="C82" s="22" t="n">
         <v>3</v>
       </c>
       <c r="D82" s="13" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E82" s="22" t="s">
         <v>335</v>
@@ -8343,16 +8352,16 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="28" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B83" s="13" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="C83" s="22" t="n">
         <v>3</v>
       </c>
       <c r="D83" s="13" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="E83" s="22" t="s">
         <v>335</v>
@@ -8363,16 +8372,16 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="28" t="s">
-        <v>171</v>
+        <v>407</v>
       </c>
       <c r="B84" s="13" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="C84" s="22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D84" s="13" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="E84" s="22" t="s">
         <v>335</v>
@@ -8383,41 +8392,61 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="28" t="s">
-        <v>407</v>
+        <v>171</v>
       </c>
       <c r="B85" s="13" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="C85" s="22" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D85" s="13" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="E85" s="22" t="s">
         <v>335</v>
       </c>
       <c r="F85" s="22" t="s">
-        <v>356</v>
+        <v>346</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="28" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B86" s="13" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="C86" s="22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D86" s="13" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="E86" s="22" t="s">
         <v>335</v>
       </c>
       <c r="F86" s="22" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="28" t="s">
+        <v>412</v>
+      </c>
+      <c r="B87" s="13" t="s">
+        <v>400</v>
+      </c>
+      <c r="C87" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D87" s="13" t="s">
+        <v>413</v>
+      </c>
+      <c r="E87" s="22" t="s">
+        <v>335</v>
+      </c>
+      <c r="F87" s="22" t="s">
         <v>346</v>
       </c>
     </row>
@@ -8457,7 +8486,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8467,7 +8496,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="4" t="n">
@@ -8479,36 +8508,36 @@
         <v>10</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>183</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="G5" s="7" t="s">
         <v>13</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="28" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="C6" s="10" t="n">
         <v>1</v>
@@ -8527,18 +8556,18 @@
         <v>17</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="I6" s="13" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="28" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="C7" s="10" t="n">
         <v>10</v>
@@ -8557,18 +8586,18 @@
         <v>18</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="I7" s="13" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="28" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="C8" s="10" t="n">
         <v>10</v>
@@ -8587,18 +8616,18 @@
         <v>19</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="I8" s="13" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="28" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="C9" s="10" t="n">
         <v>10</v>
@@ -8617,18 +8646,18 @@
         <v>17</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="I9" s="13" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="28" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="C10" s="10" t="n">
         <v>17</v>
@@ -8647,18 +8676,18 @@
         <v>18</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="I10" s="13" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="28" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="C11" s="10" t="n">
         <v>17</v>
@@ -8677,18 +8706,18 @@
         <v>17</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="I11" s="13" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="28" t="s">
+        <v>373</v>
+      </c>
+      <c r="B12" s="13" t="s">
         <v>369</v>
-      </c>
-      <c r="B12" s="13" t="s">
-        <v>365</v>
       </c>
       <c r="C12" s="10" t="n">
         <v>16</v>
@@ -8707,18 +8736,18 @@
         <v>19</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="I12" s="13" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="28" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="C13" s="10" t="n">
         <v>4</v>
@@ -8737,18 +8766,18 @@
         <v>19</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="I13" s="13" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="28" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="C14" s="10" t="n">
         <v>3</v>
@@ -8767,18 +8796,18 @@
         <v>18</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="I14" s="13" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="28" t="s">
+        <v>380</v>
+      </c>
+      <c r="B15" s="13" t="s">
         <v>376</v>
-      </c>
-      <c r="B15" s="13" t="s">
-        <v>372</v>
       </c>
       <c r="C15" s="10" t="n">
         <v>3</v>
@@ -8797,18 +8826,18 @@
         <v>17</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="I15" s="13" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="28" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="C16" s="10" t="n">
         <v>4</v>
@@ -8827,18 +8856,18 @@
         <v>19</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="I16" s="13" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="28" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="C17" s="10" t="n">
         <v>4</v>
@@ -8857,18 +8886,18 @@
         <v>19</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="I17" s="13" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="28" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="C18" s="10" t="n">
         <v>4</v>
@@ -8887,10 +8916,10 @@
         <v>19</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="I18" s="13" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8914,7 +8943,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="B21" s="14"/>
       <c r="C21" s="14"/>
@@ -8927,10 +8956,10 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="C22" s="10" t="n">
         <v>1</v>
@@ -8947,15 +8976,15 @@
         <v>168</v>
       </c>
       <c r="I22" s="8" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="C23" s="10" t="n">
         <v>1</v>
@@ -8972,15 +9001,15 @@
         <v>169</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="C24" s="10" t="n">
         <v>1</v>
@@ -8997,43 +9026,43 @@
         <v>170</v>
       </c>
       <c r="I24" s="8" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="C25" s="33" t="n">
         <f aca="false">ROUNDUP(('Kablo Çizelgesi'!K29+'Kablo Çizelgesi'!K30+'Kablo Çizelgesi'!K31)*(1+$C$3/100),0)</f>
         <v>220</v>
       </c>
       <c r="D25" s="22" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="E25" s="8"/>
       <c r="F25" s="22" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="G25" s="22" t="s">
         <v>67</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="C26" s="10" t="n">
         <v>1</v>
@@ -9047,10 +9076,10 @@
         <v>67</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="I26" s="8" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
     </row>
   </sheetData>
@@ -9086,7 +9115,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9096,7 +9125,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="4" t="n">
@@ -9105,7 +9134,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="4" t="n">
@@ -9114,7 +9143,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="4" t="n">
@@ -9123,7 +9152,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="4" t="n">
@@ -9132,7 +9161,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="4" t="n">
@@ -9141,7 +9170,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="4" t="n">
@@ -9150,7 +9179,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="4" t="n">
@@ -9159,7 +9188,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="4" t="n">
@@ -9168,7 +9197,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="4" t="n">
@@ -9177,7 +9206,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="B12" s="3"/>
       <c r="C12" s="4" t="n">
@@ -9186,7 +9215,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="4" t="n">
@@ -9195,7 +9224,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="B14" s="3"/>
       <c r="C14" s="4" t="n">
@@ -9204,7 +9233,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
       <c r="B15" s="3"/>
       <c r="C15" s="4" t="n">
@@ -9213,7 +9242,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="B16" s="3"/>
       <c r="C16" s="4" t="n">
@@ -9222,7 +9251,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="4" t="n">
@@ -9231,7 +9260,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="B18" s="3"/>
       <c r="C18" s="4" t="n">
@@ -9240,7 +9269,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="B19" s="3"/>
       <c r="C19" s="4" t="n">
@@ -9249,7 +9278,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="4" t="n">
@@ -9258,7 +9287,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="B21" s="3"/>
       <c r="C21" s="4" t="n">
@@ -9267,7 +9296,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="B22" s="3"/>
       <c r="C22" s="4" t="n">
@@ -9276,7 +9305,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="B23" s="3"/>
       <c r="C23" s="4" t="n">
@@ -9285,7 +9314,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="4" t="n">
@@ -9294,7 +9323,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="4" t="n">
@@ -9306,16 +9335,16 @@
         <v>10</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="F27" s="6" t="s">
         <v>184</v>
@@ -9323,313 +9352,313 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="28" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
       <c r="C28" s="22" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="D28" s="33" t="n">
         <f aca="false">2*(($C$3+2*$C$5)+($C$4+2*$C$5))</f>
         <v>88</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="F28" s="13" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="28" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="C29" s="22" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="D29" s="33" t="n">
         <f aca="false">ROUNDUP(D28*(1+$C$10/100),0)</f>
         <v>97</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="F29" s="13" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="28" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="C30" s="22" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="D30" s="33" t="n">
         <f aca="false">2*(ROUNDUP(($C$3+2*$C$5)/$C$8,0)+ROUNDUP(($C$4+2*$C$5)/$C$8,0))</f>
         <v>12</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="F30" s="13" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="28" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
       <c r="C31" s="22" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="D31" s="33" t="n">
         <f aca="false">D30*$C$7</f>
         <v>36</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
       <c r="F31" s="13"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="28" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="C32" s="22" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="D32" s="18" t="n">
         <f aca="false">MAX(($C$3+2*$C$5)/ROUNDUP(($C$3+2*$C$5)/$C$8,0),($C$4+2*$C$5)/ROUNDUP(($C$4+2*$C$5)/$C$8,0))</f>
         <v>7.33333333333333</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="F32" s="13" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="28" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="C33" s="22" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="D33" s="33" t="n">
         <f aca="false">$C$15</f>
         <v>4</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="F33" s="13" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="28" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="C34" s="22" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="D34" s="33" t="n">
         <f aca="false">MIN(8,MAX(2,ROUNDUP(2*($C$3+$C$4)/$C$9,0)))</f>
         <v>6</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="F34" s="13" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="28" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>502</v>
+        <v>505</v>
       </c>
       <c r="C35" s="22" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="D35" s="33" t="n">
         <f aca="false">D34</f>
         <v>6</v>
       </c>
       <c r="E35" s="13" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="F35" s="13" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="28" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="C36" s="22" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="D36" s="33" t="n">
         <f aca="false">ROUNDUP((D34*($C$11+$C$6)+($C$13-$C$11)+(PI()*$C$14/2+2))*(1+$C$10/100),0)</f>
         <v>101</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="F36" s="13" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="28" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="C37" s="22" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="D37" s="33" t="n">
         <f aca="false">ROUNDUP((2*($C$3+$C$4)+$C$4/2+3)*(1+$C$10/100),0)</f>
         <v>103</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="F37" s="13" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="28" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="C38" s="22" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="D38" s="33" t="n">
         <f aca="false">3</f>
         <v>3</v>
       </c>
       <c r="E38" s="13" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="F38" s="13" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="28" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="B39" s="13" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="C39" s="22" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="D39" s="20" t="n">
         <f aca="false">$C$23+$C$24+$C$25</f>
         <v>4.5</v>
       </c>
       <c r="E39" s="13" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="F39" s="13"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="28" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="B40" s="13" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="C40" s="22" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="D40" s="33" t="n">
         <f aca="false">1</f>
         <v>1</v>
       </c>
       <c r="E40" s="13" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="F40" s="13" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="28" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="C41" s="22" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="D41" s="33" t="n">
         <f aca="false">ROUNDUP($C$16*(1+$C$10/100),0)</f>
         <v>3</v>
       </c>
       <c r="E41" s="13" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="F41" s="13" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="28" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="C42" s="22" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="D42" s="33" t="n">
         <f aca="false">ROUNDUP($C$17*(1+$C$10/100),0)</f>
         <v>4</v>
       </c>
       <c r="E42" s="13" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="F42" s="13" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9637,167 +9666,167 @@
         <v>340</v>
       </c>
       <c r="B43" s="13" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="C43" s="22" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="D43" s="33" t="n">
         <f aca="false">ROUNDUP($C$22*(1+$C$10/100),0)</f>
         <v>33</v>
       </c>
       <c r="E43" s="13" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="F43" s="13" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="28" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="B44" s="13" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
       <c r="C44" s="22" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="D44" s="33" t="n">
         <f aca="false">$C$18</f>
         <v>3</v>
       </c>
       <c r="E44" s="13" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="F44" s="13" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="28" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="B45" s="13" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="C45" s="22" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="D45" s="33" t="n">
         <f aca="false">($C$18-1)*$C$19+6</f>
         <v>18</v>
       </c>
       <c r="E45" s="13" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="F45" s="13" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="28" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="B46" s="13" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="C46" s="22" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="D46" s="33" t="n">
         <f aca="false">ROUNDUP($C$21*$C$20*(1+$C$10/100),0)</f>
         <v>80</v>
       </c>
       <c r="E46" s="13" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="F46" s="13" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="28" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="B47" s="13" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="C47" s="22" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="D47" s="33" t="n">
         <f aca="false">$C$21</f>
         <v>6</v>
       </c>
       <c r="E47" s="13" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="F47" s="13" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="28" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="B48" s="13" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="C48" s="22" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="D48" s="33" t="n">
         <f aca="false">1</f>
         <v>1</v>
       </c>
       <c r="E48" s="13" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="F48" s="13" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="28" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="B49" s="13" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
       <c r="C49" s="22" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="D49" s="33" t="n">
         <f aca="false">D30+D34+2+1+$C$21</f>
         <v>27</v>
       </c>
       <c r="E49" s="13" t="s">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="F49" s="13" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="28" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="B50" s="13" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="C50" s="22" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="D50" s="33" t="n">
         <f aca="false">3</f>
         <v>3</v>
       </c>
       <c r="E50" s="13" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="F50" s="13" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9805,17 +9834,17 @@
         <v>67</v>
       </c>
       <c r="B51" s="13" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="C51" s="22" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="D51" s="33" t="n">
         <f aca="false">ROUNDUP(D49/10,0)</f>
         <v>3</v>
       </c>
       <c r="E51" s="13" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="F51" s="13"/>
     </row>
@@ -9877,7 +9906,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9887,7 +9916,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -9907,7 +9936,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -9917,7 +9946,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -9927,7 +9956,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
@@ -9937,7 +9966,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -9957,7 +9986,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -9967,7 +9996,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -9987,7 +10016,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -9997,7 +10026,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -10007,7 +10036,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -10017,7 +10046,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -10027,7 +10056,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -10037,7 +10066,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -10047,7 +10076,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -10057,7 +10086,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -10067,7 +10096,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="14" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="B22" s="14"/>
       <c r="C22" s="14"/>
@@ -10081,7 +10110,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -10090,12 +10119,12 @@
         <v>360.843918243516</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -10104,12 +10133,12 @@
         <v>9.0210979560879</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -10118,12 +10147,12 @@
         <v>0.0256</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
@@ -10132,12 +10161,12 @@
         <v>0.00832</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
@@ -10146,12 +10175,12 @@
         <v>0.0242102788088035</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
@@ -10160,12 +10189,12 @@
         <v>0.0056390977443609</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -10174,12 +10203,12 @@
         <v>0.0024</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
@@ -10188,12 +10217,12 @@
         <v>0.0300493485473292</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>584</v>
+        <v>587</v>
       </c>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
@@ -10202,12 +10231,12 @@
         <v>7.68536154160241</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="B33" s="14"/>
       <c r="C33" s="14"/>
@@ -10221,45 +10250,45 @@
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
       <c r="B34" s="7" t="s">
         <v>10</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="G34" s="7" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="H34" s="7" t="s">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="I34" s="7" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="J34" s="7" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="22" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="B35" s="28" t="s">
         <v>141</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>595</v>
+        <v>598</v>
       </c>
       <c r="D35" s="22" t="n">
         <f aca="false">$D$12</f>
@@ -10285,18 +10314,18 @@
         <v>UYGUN</v>
       </c>
       <c r="J35" s="13" t="s">
-        <v>596</v>
+        <v>599</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="22" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="B36" s="28" t="s">
         <v>199</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
       <c r="D36" s="22" t="s">
         <v>67</v>
@@ -10322,18 +10351,18 @@
         <v>UYGUN</v>
       </c>
       <c r="J36" s="13" t="s">
-        <v>599</v>
+        <v>602</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="22" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="B37" s="28" t="s">
         <v>273</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
       <c r="D37" s="22" t="n">
         <v>63</v>
@@ -10357,18 +10386,18 @@
         <v>UYGUN</v>
       </c>
       <c r="J37" s="13" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="22" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="B38" s="28" t="s">
         <v>240</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>603</v>
+        <v>606</v>
       </c>
       <c r="D38" s="22" t="n">
         <v>25</v>
@@ -10392,18 +10421,18 @@
         <v>UYGUN</v>
       </c>
       <c r="J38" s="13" t="s">
-        <v>604</v>
+        <v>607</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="22" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="B39" s="28" t="s">
         <v>243</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>605</v>
+        <v>608</v>
       </c>
       <c r="D39" s="22" t="n">
         <v>25</v>
@@ -10426,18 +10455,18 @@
         <v>UYGUN</v>
       </c>
       <c r="J39" s="13" t="s">
-        <v>606</v>
+        <v>609</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="22" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="B40" s="28" t="s">
         <v>276</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>607</v>
+        <v>610</v>
       </c>
       <c r="D40" s="22" t="n">
         <v>63</v>
@@ -10460,18 +10489,18 @@
         <v>UYGUN</v>
       </c>
       <c r="J40" s="13" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="22" t="s">
-        <v>609</v>
+        <v>612</v>
       </c>
       <c r="B41" s="28" t="s">
         <v>279</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>610</v>
+        <v>613</v>
       </c>
       <c r="D41" s="22" t="n">
         <v>14</v>
@@ -10498,16 +10527,16 @@
     </row>
     <row r="42" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="22" t="s">
-        <v>609</v>
+        <v>612</v>
       </c>
       <c r="B42" s="28" t="s">
-        <v>611</v>
+        <v>614</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>612</v>
+        <v>615</v>
       </c>
       <c r="D42" s="22" t="s">
-        <v>613</v>
+        <v>616</v>
       </c>
       <c r="E42" s="22" t="n">
         <v>30</v>
@@ -10527,18 +10556,18 @@
         <v>UYGUN</v>
       </c>
       <c r="J42" s="13" t="s">
-        <v>614</v>
+        <v>617</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="22" t="s">
-        <v>609</v>
+        <v>612</v>
       </c>
       <c r="B43" s="28" t="s">
         <v>282</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>615</v>
+        <v>618</v>
       </c>
       <c r="D43" s="22" t="n">
         <v>25</v>
@@ -10561,18 +10590,18 @@
         <v>UYGUN</v>
       </c>
       <c r="J43" s="13" t="s">
-        <v>616</v>
+        <v>619</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="22" t="s">
-        <v>617</v>
+        <v>620</v>
       </c>
       <c r="B44" s="28" t="s">
         <v>297</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>618</v>
+        <v>621</v>
       </c>
       <c r="D44" s="22" t="n">
         <v>10</v>
@@ -10596,15 +10625,15 @@
         <v>UYGUN</v>
       </c>
       <c r="J44" s="13" t="s">
-        <v>619</v>
+        <v>622</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="3" t="s">
-        <v>620</v>
+        <v>623</v>
       </c>
       <c r="C45" s="8" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
       <c r="G45" s="8" t="n">
         <f aca="false">$D$10</f>
@@ -10621,7 +10650,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="14" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="B47" s="14"/>
       <c r="C47" s="14"/>
@@ -10635,34 +10664,34 @@
     </row>
     <row r="48" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>624</v>
+        <v>627</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>625</v>
+        <v>628</v>
       </c>
       <c r="D48" s="7" t="s">
-        <v>626</v>
+        <v>629</v>
       </c>
       <c r="E48" s="7" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="F48" s="7" t="s">
-        <v>628</v>
+        <v>631</v>
       </c>
       <c r="G48" s="7" t="s">
-        <v>629</v>
+        <v>632</v>
       </c>
       <c r="H48" s="7" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="I48" s="7" t="s">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="J48" s="7" t="s">
-        <v>632</v>
+        <v>635</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10670,7 +10699,7 @@
         <v>199</v>
       </c>
       <c r="B49" s="13" t="s">
-        <v>633</v>
+        <v>636</v>
       </c>
       <c r="C49" s="8" t="n">
         <f aca="false">$D$15</f>
@@ -10708,7 +10737,7 @@
         <v>199</v>
       </c>
       <c r="B50" s="13" t="s">
-        <v>634</v>
+        <v>637</v>
       </c>
       <c r="C50" s="8" t="n">
         <f aca="false">$D$15</f>
@@ -10746,7 +10775,7 @@
         <v>199</v>
       </c>
       <c r="B51" s="13" t="s">
-        <v>635</v>
+        <v>638</v>
       </c>
       <c r="C51" s="8" t="n">
         <f aca="false">$D$15</f>
@@ -10781,7 +10810,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="14" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="B53" s="14"/>
       <c r="C53" s="14"/>
@@ -10795,29 +10824,29 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="6" t="s">
-        <v>637</v>
+        <v>640</v>
       </c>
       <c r="B54" s="6"/>
       <c r="C54" s="6"/>
       <c r="D54" s="6" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="F54" s="6" t="s">
-        <v>639</v>
+        <v>642</v>
       </c>
       <c r="G54" s="6"/>
       <c r="H54" s="6"/>
       <c r="I54" s="6"/>
       <c r="J54" s="6" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>640</v>
+        <v>643</v>
       </c>
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
@@ -10826,15 +10855,15 @@
         <v>960</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="J55" s="13" t="s">
-        <v>641</v>
+        <v>644</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>642</v>
+        <v>645</v>
       </c>
       <c r="B56" s="3"/>
       <c r="C56" s="3"/>
@@ -10843,19 +10872,19 @@
         <v>100</v>
       </c>
       <c r="E56" s="8" t="s">
-        <v>643</v>
+        <v>646</v>
       </c>
       <c r="F56" s="24" t="str">
         <f aca="false">IF(D56&gt;=$D$19+$D$18,"UYGUN","UYGUN DEĞİL")</f>
         <v>UYGUN</v>
       </c>
       <c r="J56" s="13" t="s">
-        <v>644</v>
+        <v>647</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="B57" s="3"/>
       <c r="C57" s="3"/>
@@ -10864,19 +10893,19 @@
         <v>10</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="F57" s="24" t="str">
         <f aca="false">IF(D57&gt;=$D$31,"UYGUN","UYGUN DEĞİL")</f>
         <v>UYGUN</v>
       </c>
       <c r="J57" s="13" t="s">
-        <v>646</v>
+        <v>649</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>647</v>
+        <v>650</v>
       </c>
       <c r="B58" s="3"/>
       <c r="C58" s="3"/>
@@ -10885,20 +10914,20 @@
         <v>7.68536154160241</v>
       </c>
       <c r="E58" s="8" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="J58" s="13" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="25" t="s">
-        <v>649</v>
+        <v>652</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="25" t="s">
-        <v>650</v>
+        <v>653</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Excel: Ses Sistemi Özeti sayfası eklendi (hoparlör, güç ve ses kablosu, ΔU, fire dahil sipariş metrajı)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NjS5sn9fPFLq7X5eqGJ5mC
</commit_message>
<xml_diff>
--- a/cikti/04_hesap_tablolari.xlsx
+++ b/cikti/04_hesap_tablolari.xlsx
@@ -12,8 +12,9 @@
     <sheet name="Kablo Çizelgesi" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Pano Malzeme Listesi" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Aydınlatma ve Priz Envanteri" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Topraklama ve Yıldırım Malzeme" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Kesici Selektivite" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Ses Sistemi Özeti" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Topraklama ve Yıldırım Malzeme" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Kesici Selektivite" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1262" uniqueCount="661">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1314" uniqueCount="690">
   <si>
     <t xml:space="preserve">YÜK DENGESİ VE FAZ DENGESİZLİĞİ</t>
   </si>
@@ -1412,6 +1413,93 @@
   </si>
   <si>
     <t xml:space="preserve">Çizim 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SES SİSTEMİ ÖZETİ (hoparlör, güç kablosu, ses kablosu; Çizim 1 ve Çizim 6 ile aynı pozlar)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kol / hat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hoparlör poz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hoparlör adedi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kol gücü (W)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Koruma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Güç kablosu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Güç kablosu L (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ΔU sonuç</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SES kablosu poz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ses kablosu tipi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ses kablosu L (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ses kablosu sipariş (m, fire dahil)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SS1 · sağ kol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W19: NYY 3x2,5 mm²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SK1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2x1,5 mm² ekranlı (LiYCY)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SS2 · sol kol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W20: NYY 3x2,5 mm²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SK2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SS3 · minare kol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W21: NYY 3x2,5 mm²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SK3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AM1 · AMF1 amfi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W18: NYY 3x2,5 mm²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SK1–SK3 (çıkışlar)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">amfi çıkışları → kol hoparlörleri</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not: Kol gücü hoparlörlere eşit bölünmüştür; amfi gücü, ses kablosu tipi ve boyları varsayımdır (sarı hücreler PARAMETRELER'den gelir). Güç kablosu uzunluğu ve ΔU değerleri 'Kablo Çizelgesi' sayfasından alınır.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ses kablosu (SK) boyları ilgili kol güç kablosu boyuyla aynı alınmıştır (varsayım); amfi çıkış tipi ve hoparlör empedans uyumu üretici verisiyle doğrulanmalıdır.</t>
   </si>
   <si>
     <t xml:space="preserve">TOPRAKLAMA VE YILDIRIMDAN KORUNMA MALZEMESİ (metraj formüllerle)</t>
@@ -2166,7 +2254,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2301,6 +2389,10 @@
     </xf>
     <xf numFmtId="168" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="169" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -3343,7 +3435,7 @@
         <v>1.93236714975845</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
         <v>49</v>
       </c>
@@ -9342,6 +9434,385 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
+  <dimension ref="A1:P13"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="4" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
+        <v>460</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>461</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>462</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>424</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>463</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>464</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>465</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>466</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>467</v>
+      </c>
+      <c r="M5" s="7" t="s">
+        <v>468</v>
+      </c>
+      <c r="N5" s="7" t="s">
+        <v>469</v>
+      </c>
+      <c r="O5" s="7" t="s">
+        <v>470</v>
+      </c>
+      <c r="P5" s="7" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="B6" s="28" t="s">
+        <v>387</v>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" s="30" t="n">
+        <f aca="false">IF(C6&gt;0,E6/C6,0)</f>
+        <v>150</v>
+      </c>
+      <c r="E6" s="30" t="n">
+        <f aca="false">'Kablo Çizelgesi'!E34*1000</f>
+        <v>600</v>
+      </c>
+      <c r="F6" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="G6" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="H6" s="13" t="s">
+        <v>473</v>
+      </c>
+      <c r="I6" s="12" t="n">
+        <f aca="false">'Kablo Çizelgesi'!K34</f>
+        <v>100</v>
+      </c>
+      <c r="J6" s="11" t="n">
+        <f aca="false">'Kablo Çizelgesi'!T34</f>
+        <v>2.3456288860756</v>
+      </c>
+      <c r="K6" s="11" t="n">
+        <f aca="false">'Kablo Çizelgesi'!U34</f>
+        <v>3</v>
+      </c>
+      <c r="L6" s="24" t="str">
+        <f aca="false">IF(J6&lt;=K6,"UYGUN","UYGUN DEĞİL")</f>
+        <v>UYGUN</v>
+      </c>
+      <c r="M6" s="31" t="s">
+        <v>474</v>
+      </c>
+      <c r="N6" s="13" t="s">
+        <v>475</v>
+      </c>
+      <c r="O6" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="P6" s="30" t="n">
+        <f aca="false">ROUNDUP(O6*(1+$C$3/100),0)</f>
+        <v>110</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>476</v>
+      </c>
+      <c r="B7" s="28" t="s">
+        <v>390</v>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" s="30" t="n">
+        <f aca="false">IF(C7&gt;0,E7/C7,0)</f>
+        <v>150</v>
+      </c>
+      <c r="E7" s="30" t="n">
+        <f aca="false">'Kablo Çizelgesi'!E35*1000</f>
+        <v>600</v>
+      </c>
+      <c r="F7" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="G7" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="H7" s="13" t="s">
+        <v>477</v>
+      </c>
+      <c r="I7" s="12" t="n">
+        <f aca="false">'Kablo Çizelgesi'!K35</f>
+        <v>100</v>
+      </c>
+      <c r="J7" s="11" t="n">
+        <f aca="false">'Kablo Çizelgesi'!T35</f>
+        <v>2.3456288860756</v>
+      </c>
+      <c r="K7" s="11" t="n">
+        <f aca="false">'Kablo Çizelgesi'!U35</f>
+        <v>3</v>
+      </c>
+      <c r="L7" s="24" t="str">
+        <f aca="false">IF(J7&lt;=K7,"UYGUN","UYGUN DEĞİL")</f>
+        <v>UYGUN</v>
+      </c>
+      <c r="M7" s="31" t="s">
+        <v>478</v>
+      </c>
+      <c r="N7" s="13" t="s">
+        <v>475</v>
+      </c>
+      <c r="O7" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="P7" s="30" t="n">
+        <f aca="false">ROUNDUP(O7*(1+$C$3/100),0)</f>
+        <v>110</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="B8" s="28" t="s">
+        <v>392</v>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" s="30" t="n">
+        <f aca="false">IF(C8&gt;0,E8/C8,0)</f>
+        <v>150</v>
+      </c>
+      <c r="E8" s="30" t="n">
+        <f aca="false">'Kablo Çizelgesi'!E36*1000</f>
+        <v>600</v>
+      </c>
+      <c r="F8" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="G8" s="13" t="s">
+        <v>167</v>
+      </c>
+      <c r="H8" s="13" t="s">
+        <v>480</v>
+      </c>
+      <c r="I8" s="12" t="n">
+        <f aca="false">'Kablo Çizelgesi'!K36</f>
+        <v>100</v>
+      </c>
+      <c r="J8" s="11" t="n">
+        <f aca="false">'Kablo Çizelgesi'!T36</f>
+        <v>2.3456288860756</v>
+      </c>
+      <c r="K8" s="11" t="n">
+        <f aca="false">'Kablo Çizelgesi'!U36</f>
+        <v>3</v>
+      </c>
+      <c r="L8" s="24" t="str">
+        <f aca="false">IF(J8&lt;=K8,"UYGUN","UYGUN DEĞİL")</f>
+        <v>UYGUN</v>
+      </c>
+      <c r="M8" s="31" t="s">
+        <v>481</v>
+      </c>
+      <c r="N8" s="13" t="s">
+        <v>475</v>
+      </c>
+      <c r="O8" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="P8" s="30" t="n">
+        <f aca="false">ROUNDUP(O8*(1+$C$3/100),0)</f>
+        <v>110</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="C9" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="30" t="n">
+        <f aca="false">E9/C9</f>
+        <v>300</v>
+      </c>
+      <c r="E9" s="30" t="n">
+        <f aca="false">'Kablo Çizelgesi'!E33*1000</f>
+        <v>300</v>
+      </c>
+      <c r="F9" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="G9" s="13" t="s">
+        <v>167</v>
+      </c>
+      <c r="H9" s="13" t="s">
+        <v>483</v>
+      </c>
+      <c r="I9" s="12" t="n">
+        <f aca="false">'Kablo Çizelgesi'!K33</f>
+        <v>5</v>
+      </c>
+      <c r="J9" s="11" t="n">
+        <f aca="false">'Kablo Çizelgesi'!T33</f>
+        <v>0.326404654435435</v>
+      </c>
+      <c r="K9" s="11" t="n">
+        <f aca="false">'Kablo Çizelgesi'!U33</f>
+        <v>3</v>
+      </c>
+      <c r="L9" s="24" t="str">
+        <f aca="false">IF(J9&lt;=K9,"UYGUN","UYGUN DEĞİL")</f>
+        <v>UYGUN</v>
+      </c>
+      <c r="M9" s="34" t="s">
+        <v>484</v>
+      </c>
+      <c r="N9" s="13" t="s">
+        <v>485</v>
+      </c>
+      <c r="O9" s="22" t="s">
+        <v>69</v>
+      </c>
+      <c r="P9" s="22" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="B10" s="15"/>
+      <c r="C10" s="32" t="n">
+        <f aca="false">SUM(C6:C8)</f>
+        <v>12</v>
+      </c>
+      <c r="D10" s="15"/>
+      <c r="E10" s="32" t="n">
+        <f aca="false">SUM(E6:E9)</f>
+        <v>2100</v>
+      </c>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="15"/>
+      <c r="I10" s="17" t="n">
+        <f aca="false">SUM(I6:I9)</f>
+        <v>305</v>
+      </c>
+      <c r="J10" s="15"/>
+      <c r="K10" s="15"/>
+      <c r="L10" s="15"/>
+      <c r="M10" s="15"/>
+      <c r="N10" s="15"/>
+      <c r="O10" s="17" t="n">
+        <f aca="false">SUM(O6:O8)</f>
+        <v>300</v>
+      </c>
+      <c r="P10" s="32" t="n">
+        <f aca="false">SUM(P6:P8)</f>
+        <v>330</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="25" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="25" t="s">
+        <v>487</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:B3"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
   <dimension ref="A1:F51"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -9355,7 +9826,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>459</v>
+        <v>488</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9365,7 +9836,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>460</v>
+        <v>489</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="4" t="n">
@@ -9374,7 +9845,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>461</v>
+        <v>490</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="4" t="n">
@@ -9383,7 +9854,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>462</v>
+        <v>491</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="4" t="n">
@@ -9392,7 +9863,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>463</v>
+        <v>492</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="4" t="n">
@@ -9401,7 +9872,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>464</v>
+        <v>493</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="4" t="n">
@@ -9410,7 +9881,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>465</v>
+        <v>494</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="4" t="n">
@@ -9419,7 +9890,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>466</v>
+        <v>495</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="4" t="n">
@@ -9428,7 +9899,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>467</v>
+        <v>496</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="4" t="n">
@@ -9437,7 +9908,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>468</v>
+        <v>497</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="4" t="n">
@@ -9446,7 +9917,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>469</v>
+        <v>498</v>
       </c>
       <c r="B12" s="3"/>
       <c r="C12" s="4" t="n">
@@ -9455,7 +9926,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>470</v>
+        <v>499</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="4" t="n">
@@ -9464,7 +9935,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>471</v>
+        <v>500</v>
       </c>
       <c r="B14" s="3"/>
       <c r="C14" s="4" t="n">
@@ -9473,7 +9944,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>472</v>
+        <v>501</v>
       </c>
       <c r="B15" s="3"/>
       <c r="C15" s="4" t="n">
@@ -9482,7 +9953,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>473</v>
+        <v>502</v>
       </c>
       <c r="B16" s="3"/>
       <c r="C16" s="4" t="n">
@@ -9491,7 +9962,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>474</v>
+        <v>503</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="4" t="n">
@@ -9500,7 +9971,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>475</v>
+        <v>504</v>
       </c>
       <c r="B18" s="3"/>
       <c r="C18" s="4" t="n">
@@ -9509,7 +9980,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>476</v>
+        <v>505</v>
       </c>
       <c r="B19" s="3"/>
       <c r="C19" s="4" t="n">
@@ -9518,7 +9989,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>477</v>
+        <v>506</v>
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="4" t="n">
@@ -9527,7 +9998,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>478</v>
+        <v>507</v>
       </c>
       <c r="B21" s="3"/>
       <c r="C21" s="4" t="n">
@@ -9536,7 +10007,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>479</v>
+        <v>508</v>
       </c>
       <c r="B22" s="3"/>
       <c r="C22" s="4" t="n">
@@ -9545,7 +10016,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>480</v>
+        <v>509</v>
       </c>
       <c r="B23" s="3"/>
       <c r="C23" s="4" t="n">
@@ -9554,7 +10025,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>481</v>
+        <v>510</v>
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="4" t="n">
@@ -9563,7 +10034,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>482</v>
+        <v>511</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="4" t="n">
@@ -9575,16 +10046,16 @@
         <v>10</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>483</v>
+        <v>512</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>484</v>
+        <v>513</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>485</v>
+        <v>514</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>486</v>
+        <v>515</v>
       </c>
       <c r="F27" s="6" t="s">
         <v>187</v>
@@ -9592,10 +10063,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="28" t="s">
-        <v>487</v>
+        <v>516</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>488</v>
+        <v>517</v>
       </c>
       <c r="C28" s="22" t="s">
         <v>452</v>
@@ -9605,18 +10076,18 @@
         <v>88</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>489</v>
+        <v>518</v>
       </c>
       <c r="F28" s="13" t="s">
-        <v>490</v>
+        <v>519</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="28" t="s">
-        <v>487</v>
+        <v>516</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>491</v>
+        <v>520</v>
       </c>
       <c r="C29" s="22" t="s">
         <v>452</v>
@@ -9626,39 +10097,39 @@
         <v>97</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>492</v>
+        <v>521</v>
       </c>
       <c r="F29" s="13" t="s">
-        <v>490</v>
+        <v>519</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="28" t="s">
-        <v>493</v>
+        <v>522</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>494</v>
+        <v>523</v>
       </c>
       <c r="C30" s="22" t="s">
-        <v>495</v>
+        <v>524</v>
       </c>
       <c r="D30" s="33" t="n">
         <f aca="false">2*(ROUNDUP(($C$3+2*$C$5)/$C$8,0)+ROUNDUP(($C$4+2*$C$5)/$C$8,0))</f>
         <v>12</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>496</v>
+        <v>525</v>
       </c>
       <c r="F30" s="13" t="s">
-        <v>497</v>
+        <v>526</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="28" t="s">
-        <v>493</v>
+        <v>522</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>498</v>
+        <v>527</v>
       </c>
       <c r="C31" s="22" t="s">
         <v>452</v>
@@ -9668,16 +10139,16 @@
         <v>36</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>499</v>
+        <v>528</v>
       </c>
       <c r="F31" s="13"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="28" t="s">
-        <v>493</v>
+        <v>522</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>500</v>
+        <v>529</v>
       </c>
       <c r="C32" s="22" t="s">
         <v>452</v>
@@ -9687,81 +10158,81 @@
         <v>7.33333333333333</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>501</v>
+        <v>530</v>
       </c>
       <c r="F32" s="13" t="s">
-        <v>502</v>
+        <v>531</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="28" t="s">
-        <v>503</v>
+        <v>532</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>504</v>
+        <v>533</v>
       </c>
       <c r="C33" s="22" t="s">
-        <v>495</v>
+        <v>524</v>
       </c>
       <c r="D33" s="33" t="n">
         <f aca="false">$C$15</f>
         <v>4</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>505</v>
+        <v>534</v>
       </c>
       <c r="F33" s="13" t="s">
-        <v>506</v>
+        <v>535</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="28" t="s">
-        <v>507</v>
+        <v>536</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>508</v>
+        <v>537</v>
       </c>
       <c r="C34" s="22" t="s">
-        <v>495</v>
+        <v>524</v>
       </c>
       <c r="D34" s="33" t="n">
         <f aca="false">MIN(8,MAX(2,ROUNDUP(2*($C$3+$C$4)/$C$9,0)))</f>
         <v>6</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>509</v>
+        <v>538</v>
       </c>
       <c r="F34" s="13" t="s">
-        <v>510</v>
+        <v>539</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="28" t="s">
-        <v>511</v>
+        <v>540</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>512</v>
+        <v>541</v>
       </c>
       <c r="C35" s="22" t="s">
-        <v>495</v>
+        <v>524</v>
       </c>
       <c r="D35" s="33" t="n">
         <f aca="false">D34</f>
         <v>6</v>
       </c>
       <c r="E35" s="13" t="s">
-        <v>513</v>
+        <v>542</v>
       </c>
       <c r="F35" s="13" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="28" t="s">
-        <v>507</v>
+        <v>536</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="C36" s="22" t="s">
         <v>452</v>
@@ -9771,18 +10242,18 @@
         <v>101</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>516</v>
+        <v>545</v>
       </c>
       <c r="F36" s="13" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="28" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>519</v>
+        <v>548</v>
       </c>
       <c r="C37" s="22" t="s">
         <v>452</v>
@@ -9792,39 +10263,39 @@
         <v>103</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>520</v>
+        <v>549</v>
       </c>
       <c r="F37" s="13" t="s">
-        <v>521</v>
+        <v>550</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="28" t="s">
-        <v>522</v>
+        <v>551</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>523</v>
+        <v>552</v>
       </c>
       <c r="C38" s="22" t="s">
-        <v>495</v>
+        <v>524</v>
       </c>
       <c r="D38" s="33" t="n">
         <f aca="false">3</f>
         <v>3</v>
       </c>
       <c r="E38" s="13" t="s">
-        <v>524</v>
+        <v>553</v>
       </c>
       <c r="F38" s="13" t="s">
-        <v>525</v>
+        <v>554</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="28" t="s">
-        <v>522</v>
+        <v>551</v>
       </c>
       <c r="B39" s="13" t="s">
-        <v>526</v>
+        <v>555</v>
       </c>
       <c r="C39" s="22" t="s">
         <v>452</v>
@@ -9834,37 +10305,37 @@
         <v>4.5</v>
       </c>
       <c r="E39" s="13" t="s">
-        <v>527</v>
+        <v>556</v>
       </c>
       <c r="F39" s="13"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="28" t="s">
-        <v>528</v>
+        <v>557</v>
       </c>
       <c r="B40" s="13" t="s">
-        <v>529</v>
+        <v>558</v>
       </c>
       <c r="C40" s="22" t="s">
-        <v>495</v>
+        <v>524</v>
       </c>
       <c r="D40" s="33" t="n">
         <f aca="false">1</f>
         <v>1</v>
       </c>
       <c r="E40" s="13" t="s">
-        <v>530</v>
+        <v>559</v>
       </c>
       <c r="F40" s="13" t="s">
-        <v>531</v>
+        <v>560</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="28" t="s">
-        <v>532</v>
+        <v>561</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>533</v>
+        <v>562</v>
       </c>
       <c r="C41" s="22" t="s">
         <v>452</v>
@@ -9874,18 +10345,18 @@
         <v>3</v>
       </c>
       <c r="E41" s="13" t="s">
-        <v>534</v>
+        <v>563</v>
       </c>
       <c r="F41" s="13" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="28" t="s">
-        <v>535</v>
+        <v>564</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>536</v>
+        <v>565</v>
       </c>
       <c r="C42" s="22" t="s">
         <v>452</v>
@@ -9895,10 +10366,10 @@
         <v>4</v>
       </c>
       <c r="E42" s="13" t="s">
-        <v>534</v>
+        <v>563</v>
       </c>
       <c r="F42" s="13" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9906,7 +10377,7 @@
         <v>343</v>
       </c>
       <c r="B43" s="13" t="s">
-        <v>537</v>
+        <v>566</v>
       </c>
       <c r="C43" s="22" t="s">
         <v>452</v>
@@ -9916,39 +10387,39 @@
         <v>33</v>
       </c>
       <c r="E43" s="13" t="s">
-        <v>538</v>
+        <v>567</v>
       </c>
       <c r="F43" s="13" t="s">
-        <v>539</v>
+        <v>568</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="28" t="s">
-        <v>540</v>
+        <v>569</v>
       </c>
       <c r="B44" s="13" t="s">
-        <v>541</v>
+        <v>570</v>
       </c>
       <c r="C44" s="22" t="s">
-        <v>495</v>
+        <v>524</v>
       </c>
       <c r="D44" s="33" t="n">
         <f aca="false">$C$18</f>
         <v>3</v>
       </c>
       <c r="E44" s="13" t="s">
-        <v>505</v>
+        <v>534</v>
       </c>
       <c r="F44" s="13" t="s">
-        <v>542</v>
+        <v>571</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="28" t="s">
-        <v>540</v>
+        <v>569</v>
       </c>
       <c r="B45" s="13" t="s">
-        <v>543</v>
+        <v>572</v>
       </c>
       <c r="C45" s="22" t="s">
         <v>452</v>
@@ -9958,18 +10429,18 @@
         <v>18</v>
       </c>
       <c r="E45" s="13" t="s">
-        <v>544</v>
+        <v>573</v>
       </c>
       <c r="F45" s="13" t="s">
-        <v>545</v>
+        <v>574</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="28" t="s">
-        <v>546</v>
+        <v>575</v>
       </c>
       <c r="B46" s="13" t="s">
-        <v>547</v>
+        <v>576</v>
       </c>
       <c r="C46" s="22" t="s">
         <v>452</v>
@@ -9979,94 +10450,94 @@
         <v>80</v>
       </c>
       <c r="E46" s="13" t="s">
-        <v>548</v>
+        <v>577</v>
       </c>
       <c r="F46" s="13" t="s">
-        <v>549</v>
+        <v>578</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="28" t="s">
-        <v>546</v>
+        <v>575</v>
       </c>
       <c r="B47" s="13" t="s">
-        <v>550</v>
+        <v>579</v>
       </c>
       <c r="C47" s="22" t="s">
-        <v>495</v>
+        <v>524</v>
       </c>
       <c r="D47" s="33" t="n">
         <f aca="false">$C$21</f>
         <v>6</v>
       </c>
       <c r="E47" s="13" t="s">
-        <v>551</v>
+        <v>580</v>
       </c>
       <c r="F47" s="13" t="s">
-        <v>552</v>
+        <v>581</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="28" t="s">
-        <v>553</v>
+        <v>582</v>
       </c>
       <c r="B48" s="13" t="s">
-        <v>554</v>
+        <v>583</v>
       </c>
       <c r="C48" s="22" t="s">
-        <v>495</v>
+        <v>524</v>
       </c>
       <c r="D48" s="33" t="n">
         <f aca="false">1</f>
         <v>1</v>
       </c>
       <c r="E48" s="13" t="s">
-        <v>555</v>
+        <v>584</v>
       </c>
       <c r="F48" s="13" t="s">
-        <v>556</v>
+        <v>585</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="28" t="s">
-        <v>557</v>
+        <v>586</v>
       </c>
       <c r="B49" s="13" t="s">
-        <v>558</v>
+        <v>587</v>
       </c>
       <c r="C49" s="22" t="s">
-        <v>495</v>
+        <v>524</v>
       </c>
       <c r="D49" s="33" t="n">
         <f aca="false">D30+D34+2+1+$C$21</f>
         <v>27</v>
       </c>
       <c r="E49" s="13" t="s">
-        <v>559</v>
+        <v>588</v>
       </c>
       <c r="F49" s="13" t="s">
-        <v>560</v>
+        <v>589</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="28" t="s">
-        <v>557</v>
+        <v>586</v>
       </c>
       <c r="B50" s="13" t="s">
-        <v>561</v>
+        <v>590</v>
       </c>
       <c r="C50" s="22" t="s">
-        <v>495</v>
+        <v>524</v>
       </c>
       <c r="D50" s="33" t="n">
         <f aca="false">3</f>
         <v>3</v>
       </c>
       <c r="E50" s="13" t="s">
-        <v>562</v>
+        <v>591</v>
       </c>
       <c r="F50" s="13" t="s">
-        <v>563</v>
+        <v>592</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10074,17 +10545,17 @@
         <v>69</v>
       </c>
       <c r="B51" s="13" t="s">
-        <v>564</v>
+        <v>593</v>
       </c>
       <c r="C51" s="22" t="s">
-        <v>495</v>
+        <v>524</v>
       </c>
       <c r="D51" s="33" t="n">
         <f aca="false">ROUNDUP(D49/10,0)</f>
         <v>3</v>
       </c>
       <c r="E51" s="13" t="s">
-        <v>565</v>
+        <v>594</v>
       </c>
       <c r="F51" s="13"/>
     </row>
@@ -10124,7 +10595,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
@@ -10146,7 +10617,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>566</v>
+        <v>595</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10156,7 +10627,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>567</v>
+        <v>596</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -10176,7 +10647,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>568</v>
+        <v>597</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -10186,7 +10657,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>569</v>
+        <v>598</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -10196,7 +10667,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>570</v>
+        <v>599</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
@@ -10206,7 +10677,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>571</v>
+        <v>600</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -10226,7 +10697,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>572</v>
+        <v>601</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -10236,7 +10707,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>573</v>
+        <v>602</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -10256,7 +10727,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>574</v>
+        <v>603</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -10266,7 +10737,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>575</v>
+        <v>604</v>
       </c>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -10276,7 +10747,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>576</v>
+        <v>605</v>
       </c>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -10286,7 +10757,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>577</v>
+        <v>606</v>
       </c>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -10296,7 +10767,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>578</v>
+        <v>607</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -10306,7 +10777,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>579</v>
+        <v>608</v>
       </c>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -10316,7 +10787,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>580</v>
+        <v>609</v>
       </c>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -10326,7 +10797,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>581</v>
+        <v>610</v>
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -10336,7 +10807,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="14" t="s">
-        <v>582</v>
+        <v>611</v>
       </c>
       <c r="B22" s="14"/>
       <c r="C22" s="14"/>
@@ -10350,7 +10821,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>583</v>
+        <v>612</v>
       </c>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -10359,12 +10830,12 @@
         <v>360.843918243516</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>584</v>
+        <v>613</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>585</v>
+        <v>614</v>
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -10373,96 +10844,96 @@
         <v>9.0210979560879</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>586</v>
+        <v>615</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>587</v>
+        <v>616</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
-      <c r="D25" s="34" t="n">
+      <c r="D25" s="35" t="n">
         <f aca="false">$D$5/100*$D$4^2/($D$3*1000)</f>
         <v>0.0256</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>588</v>
+        <v>617</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>589</v>
+        <v>618</v>
       </c>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
-      <c r="D26" s="34" t="n">
+      <c r="D26" s="35" t="n">
         <f aca="false">$D$6/100*$D$4^2/($D$3*1000)</f>
         <v>0.00832</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>588</v>
+        <v>617</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>590</v>
+        <v>619</v>
       </c>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
-      <c r="D27" s="34" t="n">
+      <c r="D27" s="35" t="n">
         <f aca="false">SQRT($D$25^2-$D$26^2)</f>
         <v>0.0242102788088035</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>588</v>
+        <v>617</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>591</v>
+        <v>620</v>
       </c>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
-      <c r="D28" s="34" t="n">
+      <c r="D28" s="35" t="n">
         <f aca="false">$D$7/(56*$D$8)</f>
         <v>0.0056390977443609</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>588</v>
+        <v>617</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>592</v>
+        <v>621</v>
       </c>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
-      <c r="D29" s="34" t="n">
+      <c r="D29" s="35" t="n">
         <f aca="false">$D$9/1000*$D$7</f>
         <v>0.0024</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>588</v>
+        <v>617</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>593</v>
+        <v>622</v>
       </c>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
-      <c r="D30" s="34" t="n">
+      <c r="D30" s="35" t="n">
         <f aca="false">SQRT(($D$26+$D$28)^2+($D$27+$D$29)^2)</f>
         <v>0.0300493485473292</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>588</v>
+        <v>617</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>594</v>
+        <v>623</v>
       </c>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
@@ -10471,12 +10942,12 @@
         <v>7.68536154160241</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>586</v>
+        <v>615</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="s">
-        <v>595</v>
+        <v>624</v>
       </c>
       <c r="B33" s="14"/>
       <c r="C33" s="14"/>
@@ -10490,31 +10961,31 @@
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>596</v>
+        <v>625</v>
       </c>
       <c r="B34" s="7" t="s">
         <v>10</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>597</v>
+        <v>626</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>598</v>
+        <v>627</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>599</v>
+        <v>628</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>600</v>
+        <v>629</v>
       </c>
       <c r="G34" s="7" t="s">
-        <v>601</v>
+        <v>630</v>
       </c>
       <c r="H34" s="7" t="s">
-        <v>602</v>
+        <v>631</v>
       </c>
       <c r="I34" s="7" t="s">
-        <v>603</v>
+        <v>632</v>
       </c>
       <c r="J34" s="7" t="s">
         <v>428</v>
@@ -10522,13 +10993,13 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="22" t="s">
-        <v>604</v>
+        <v>633</v>
       </c>
       <c r="B35" s="28" t="s">
         <v>143</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>605</v>
+        <v>634</v>
       </c>
       <c r="D35" s="22" t="n">
         <f aca="false">$D$12</f>
@@ -10554,18 +11025,18 @@
         <v>UYGUN</v>
       </c>
       <c r="J35" s="13" t="s">
-        <v>606</v>
+        <v>635</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="22" t="s">
-        <v>607</v>
+        <v>636</v>
       </c>
       <c r="B36" s="28" t="s">
         <v>202</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>608</v>
+        <v>637</v>
       </c>
       <c r="D36" s="22" t="s">
         <v>69</v>
@@ -10591,18 +11062,18 @@
         <v>UYGUN</v>
       </c>
       <c r="J36" s="13" t="s">
-        <v>609</v>
+        <v>638</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="22" t="s">
-        <v>610</v>
+        <v>639</v>
       </c>
       <c r="B37" s="28" t="s">
         <v>276</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>611</v>
+        <v>640</v>
       </c>
       <c r="D37" s="22" t="n">
         <v>63</v>
@@ -10626,18 +11097,18 @@
         <v>UYGUN</v>
       </c>
       <c r="J37" s="13" t="s">
-        <v>612</v>
+        <v>641</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="22" t="s">
-        <v>610</v>
+        <v>639</v>
       </c>
       <c r="B38" s="28" t="s">
         <v>243</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>613</v>
+        <v>642</v>
       </c>
       <c r="D38" s="22" t="n">
         <v>25</v>
@@ -10661,18 +11132,18 @@
         <v>UYGUN</v>
       </c>
       <c r="J38" s="13" t="s">
-        <v>614</v>
+        <v>643</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="22" t="s">
-        <v>610</v>
+        <v>639</v>
       </c>
       <c r="B39" s="28" t="s">
         <v>246</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>615</v>
+        <v>644</v>
       </c>
       <c r="D39" s="22" t="n">
         <v>25</v>
@@ -10695,18 +11166,18 @@
         <v>UYGUN</v>
       </c>
       <c r="J39" s="13" t="s">
-        <v>616</v>
+        <v>645</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="22" t="s">
-        <v>610</v>
+        <v>639</v>
       </c>
       <c r="B40" s="28" t="s">
         <v>279</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>617</v>
+        <v>646</v>
       </c>
       <c r="D40" s="22" t="n">
         <v>63</v>
@@ -10729,18 +11200,18 @@
         <v>UYGUN</v>
       </c>
       <c r="J40" s="13" t="s">
-        <v>618</v>
+        <v>647</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="22" t="s">
-        <v>619</v>
+        <v>648</v>
       </c>
       <c r="B41" s="28" t="s">
         <v>282</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>620</v>
+        <v>649</v>
       </c>
       <c r="D41" s="22" t="n">
         <v>14</v>
@@ -10767,16 +11238,16 @@
     </row>
     <row r="42" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="22" t="s">
-        <v>619</v>
+        <v>648</v>
       </c>
       <c r="B42" s="28" t="s">
-        <v>621</v>
+        <v>650</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>622</v>
+        <v>651</v>
       </c>
       <c r="D42" s="22" t="s">
-        <v>623</v>
+        <v>652</v>
       </c>
       <c r="E42" s="22" t="n">
         <v>30</v>
@@ -10796,18 +11267,18 @@
         <v>UYGUN</v>
       </c>
       <c r="J42" s="13" t="s">
-        <v>624</v>
+        <v>653</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="22" t="s">
-        <v>619</v>
+        <v>648</v>
       </c>
       <c r="B43" s="28" t="s">
         <v>285</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>625</v>
+        <v>654</v>
       </c>
       <c r="D43" s="22" t="n">
         <v>25</v>
@@ -10830,18 +11301,18 @@
         <v>UYGUN</v>
       </c>
       <c r="J43" s="13" t="s">
-        <v>626</v>
+        <v>655</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="22" t="s">
-        <v>627</v>
+        <v>656</v>
       </c>
       <c r="B44" s="28" t="s">
         <v>301</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>628</v>
+        <v>657</v>
       </c>
       <c r="D44" s="22" t="n">
         <v>10</v>
@@ -10865,15 +11336,15 @@
         <v>UYGUN</v>
       </c>
       <c r="J44" s="13" t="s">
-        <v>629</v>
+        <v>658</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="3" t="s">
-        <v>630</v>
+        <v>659</v>
       </c>
       <c r="C45" s="8" t="s">
-        <v>631</v>
+        <v>660</v>
       </c>
       <c r="G45" s="8" t="n">
         <f aca="false">$D$10</f>
@@ -10890,7 +11361,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="14" t="s">
-        <v>632</v>
+        <v>661</v>
       </c>
       <c r="B47" s="14"/>
       <c r="C47" s="14"/>
@@ -10904,34 +11375,34 @@
     </row>
     <row r="48" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
-        <v>633</v>
+        <v>662</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>634</v>
+        <v>663</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>635</v>
+        <v>664</v>
       </c>
       <c r="D48" s="7" t="s">
-        <v>636</v>
+        <v>665</v>
       </c>
       <c r="E48" s="7" t="s">
-        <v>637</v>
+        <v>666</v>
       </c>
       <c r="F48" s="7" t="s">
-        <v>638</v>
+        <v>667</v>
       </c>
       <c r="G48" s="7" t="s">
-        <v>639</v>
+        <v>668</v>
       </c>
       <c r="H48" s="7" t="s">
-        <v>640</v>
+        <v>669</v>
       </c>
       <c r="I48" s="7" t="s">
-        <v>641</v>
+        <v>670</v>
       </c>
       <c r="J48" s="7" t="s">
-        <v>642</v>
+        <v>671</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10939,7 +11410,7 @@
         <v>202</v>
       </c>
       <c r="B49" s="13" t="s">
-        <v>643</v>
+        <v>672</v>
       </c>
       <c r="C49" s="8" t="n">
         <f aca="false">$D$15</f>
@@ -10977,7 +11448,7 @@
         <v>202</v>
       </c>
       <c r="B50" s="13" t="s">
-        <v>644</v>
+        <v>673</v>
       </c>
       <c r="C50" s="8" t="n">
         <f aca="false">$D$15</f>
@@ -11015,7 +11486,7 @@
         <v>202</v>
       </c>
       <c r="B51" s="13" t="s">
-        <v>645</v>
+        <v>674</v>
       </c>
       <c r="C51" s="8" t="n">
         <f aca="false">$D$15</f>
@@ -11050,7 +11521,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="14" t="s">
-        <v>646</v>
+        <v>675</v>
       </c>
       <c r="B53" s="14"/>
       <c r="C53" s="14"/>
@@ -11064,18 +11535,18 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="6" t="s">
-        <v>647</v>
+        <v>676</v>
       </c>
       <c r="B54" s="6"/>
       <c r="C54" s="6"/>
       <c r="D54" s="6" t="s">
-        <v>648</v>
+        <v>677</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>484</v>
+        <v>513</v>
       </c>
       <c r="F54" s="6" t="s">
-        <v>649</v>
+        <v>678</v>
       </c>
       <c r="G54" s="6"/>
       <c r="H54" s="6"/>
@@ -11086,7 +11557,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>650</v>
+        <v>679</v>
       </c>
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
@@ -11095,15 +11566,15 @@
         <v>960</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>584</v>
+        <v>613</v>
       </c>
       <c r="J55" s="13" t="s">
-        <v>651</v>
+        <v>680</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>652</v>
+        <v>681</v>
       </c>
       <c r="B56" s="3"/>
       <c r="C56" s="3"/>
@@ -11112,19 +11583,19 @@
         <v>100</v>
       </c>
       <c r="E56" s="8" t="s">
-        <v>653</v>
+        <v>682</v>
       </c>
       <c r="F56" s="24" t="str">
         <f aca="false">IF(D56&gt;=$D$19+$D$18,"UYGUN","UYGUN DEĞİL")</f>
         <v>UYGUN</v>
       </c>
       <c r="J56" s="13" t="s">
-        <v>654</v>
+        <v>683</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
-        <v>655</v>
+        <v>684</v>
       </c>
       <c r="B57" s="3"/>
       <c r="C57" s="3"/>
@@ -11133,19 +11604,19 @@
         <v>10</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>586</v>
+        <v>615</v>
       </c>
       <c r="F57" s="24" t="str">
         <f aca="false">IF(D57&gt;=$D$31,"UYGUN","UYGUN DEĞİL")</f>
         <v>UYGUN</v>
       </c>
       <c r="J57" s="13" t="s">
-        <v>656</v>
+        <v>685</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>657</v>
+        <v>686</v>
       </c>
       <c r="B58" s="3"/>
       <c r="C58" s="3"/>
@@ -11154,20 +11625,20 @@
         <v>7.68536154160241</v>
       </c>
       <c r="E58" s="8" t="s">
-        <v>586</v>
+        <v>615</v>
       </c>
       <c r="J58" s="13" t="s">
-        <v>658</v>
+        <v>687</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="25" t="s">
-        <v>659</v>
+        <v>688</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="25" t="s">
-        <v>660</v>
+        <v>689</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Çizim 3: ses kollarının topraklaması (PE damarı, EB7 amfi/SK ekran barası, EB8 minare ses grubu) eklendi
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NjS5sn9fPFLq7X5eqGJ5mC
</commit_message>
<xml_diff>
--- a/cikti/04_hesap_tablolari.xlsx
+++ b/cikti/04_hesap_tablolari.xlsx
@@ -1763,7 +1763,7 @@
     <t xml:space="preserve">50 mm² Cu çıplak</t>
   </si>
   <si>
-    <t xml:space="preserve">EB1–EB6</t>
+    <t xml:space="preserve">EB1–EB8</t>
   </si>
   <si>
     <t xml:space="preserve">Eş potansiyel bağlantı iletkeni 16 mm² Cu (sarı-yeşil)</t>
@@ -10002,7 +10002,7 @@
       </c>
       <c r="B21" s="3"/>
       <c r="C21" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10447,7 +10447,7 @@
       </c>
       <c r="D46" s="33" t="n">
         <f aca="false">ROUNDUP($C$21*$C$20*(1+$C$10/100),0)</f>
-        <v>80</v>
+        <v>106</v>
       </c>
       <c r="E46" s="13" t="s">
         <v>577</v>
@@ -10468,7 +10468,7 @@
       </c>
       <c r="D47" s="33" t="n">
         <f aca="false">$C$21</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E47" s="13" t="s">
         <v>580</v>
@@ -10510,7 +10510,7 @@
       </c>
       <c r="D49" s="33" t="n">
         <f aca="false">D30+D34+2+1+$C$21</f>
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E49" s="13" t="s">
         <v>588</v>

</xml_diff>

<commit_message>
Çıktıların Türkmen dili kopyası (tm/): çeviri sözlüğü, tm çizimleri, Excel, rapor ve README
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NjS5sn9fPFLq7X5eqGJ5mC
</commit_message>
<xml_diff>
--- a/cikti/04_hesap_tablolari.xlsx
+++ b/cikti/04_hesap_tablolari.xlsx
@@ -3387,7 +3387,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
         <v>47</v>
       </c>
@@ -3435,7 +3435,7 @@
         <v>1.93236714975845</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
         <v>49</v>
       </c>
@@ -6044,7 +6044,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
         <v>168</v>
       </c>
@@ -6204,7 +6204,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
         <v>170</v>
       </c>

</xml_diff>

<commit_message>
Türkmen README: parametre listesi ve ses sistemi parametreleri eklendi
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NjS5sn9fPFLq7X5eqGJ5mC
</commit_message>
<xml_diff>
--- a/cikti/04_hesap_tablolari.xlsx
+++ b/cikti/04_hesap_tablolari.xlsx
@@ -3387,7 +3387,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
         <v>47</v>
       </c>
@@ -3435,7 +3435,7 @@
         <v>1.93236714975845</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
         <v>49</v>
       </c>
@@ -6044,7 +6044,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
         <v>168</v>
       </c>
@@ -6204,7 +6204,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
         <v>170</v>
       </c>

</xml_diff>